<commit_message>
1998 előtti GYES kezelése bér nélkül
</commit_message>
<xml_diff>
--- a/solutions/tools/tvSearch/idovonal/szolgalatiIdok.xlsx
+++ b/solutions/tools/tvSearch/idovonal/szolgalatiIdok.xlsx
@@ -9418,7 +9418,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Gyermekes jogcím.</t>
+          <t>Gyermekes jogcím. 1998.01.01 ELŐTT: alanyi jogú biztosítás – szolgálati idő elfogadható, bér/járulék NEM vizsgálható (elfogadott_bér = 0). 1998.01.01-TŐL: nyugdíjjárulék levonásra kerül a GYES összegéből → járulékalap elfogadható.</t>
         </is>
       </c>
     </row>
@@ -12399,7 +12399,7 @@
         <v/>
       </c>
       <c r="AH5" s="6">
-        <f>IF(S5="","",IF(OR(I5=0,V5="IGEN",W5="IGEN"),0,IF(AND(K5&lt;&gt;"IGEN",L5="IGEN",U5="NEM"),0,S5)))</f>
+        <f>IF(S5="","",IF(OR(I5=0,V5="IGEN",W5="IGEN"),0,IF(AND(K5&lt;&gt;"IGEN",L5="IGEN",U5="NEM"),0,IF(AND(H5="GYES",E5&lt;1998),0,S5))))</f>
         <v/>
       </c>
       <c r="AI5" s="6">
@@ -12519,7 +12519,7 @@
         <v/>
       </c>
       <c r="AH6" s="6">
-        <f>IF(S6="","",IF(OR(I6=0,V6="IGEN",W6="IGEN"),0,IF(AND(K6&lt;&gt;"IGEN",L6="IGEN",U6="NEM"),0,S6)))</f>
+        <f>IF(S6="","",IF(OR(I6=0,V6="IGEN",W6="IGEN"),0,IF(AND(K6&lt;&gt;"IGEN",L6="IGEN",U6="NEM"),0,IF(AND(H6="GYES",E6&lt;1998),0,S6))))</f>
         <v/>
       </c>
       <c r="AI6" s="6">
@@ -12639,7 +12639,7 @@
         <v/>
       </c>
       <c r="AH7" s="6">
-        <f>IF(S7="","",IF(OR(I7=0,V7="IGEN",W7="IGEN"),0,IF(AND(K7&lt;&gt;"IGEN",L7="IGEN",U7="NEM"),0,S7)))</f>
+        <f>IF(S7="","",IF(OR(I7=0,V7="IGEN",W7="IGEN"),0,IF(AND(K7&lt;&gt;"IGEN",L7="IGEN",U7="NEM"),0,IF(AND(H7="GYES",E7&lt;1998),0,S7))))</f>
         <v/>
       </c>
       <c r="AI7" s="6">
@@ -12759,7 +12759,7 @@
         <v/>
       </c>
       <c r="AH8" s="6">
-        <f>IF(S8="","",IF(OR(I8=0,V8="IGEN",W8="IGEN"),0,IF(AND(K8&lt;&gt;"IGEN",L8="IGEN",U8="NEM"),0,S8)))</f>
+        <f>IF(S8="","",IF(OR(I8=0,V8="IGEN",W8="IGEN"),0,IF(AND(K8&lt;&gt;"IGEN",L8="IGEN",U8="NEM"),0,IF(AND(H8="GYES",E8&lt;1998),0,S8))))</f>
         <v/>
       </c>
       <c r="AI8" s="6">
@@ -12879,7 +12879,7 @@
         <v/>
       </c>
       <c r="AH9" s="6">
-        <f>IF(S9="","",IF(OR(I9=0,V9="IGEN",W9="IGEN"),0,IF(AND(K9&lt;&gt;"IGEN",L9="IGEN",U9="NEM"),0,S9)))</f>
+        <f>IF(S9="","",IF(OR(I9=0,V9="IGEN",W9="IGEN"),0,IF(AND(K9&lt;&gt;"IGEN",L9="IGEN",U9="NEM"),0,IF(AND(H9="GYES",E9&lt;1998),0,S9))))</f>
         <v/>
       </c>
       <c r="AI9" s="6">
@@ -12999,7 +12999,7 @@
         <v/>
       </c>
       <c r="AH10" s="6">
-        <f>IF(S10="","",IF(OR(I10=0,V10="IGEN",W10="IGEN"),0,IF(AND(K10&lt;&gt;"IGEN",L10="IGEN",U10="NEM"),0,S10)))</f>
+        <f>IF(S10="","",IF(OR(I10=0,V10="IGEN",W10="IGEN"),0,IF(AND(K10&lt;&gt;"IGEN",L10="IGEN",U10="NEM"),0,IF(AND(H10="GYES",E10&lt;1998),0,S10))))</f>
         <v/>
       </c>
       <c r="AI10" s="6">
@@ -13119,7 +13119,7 @@
         <v/>
       </c>
       <c r="AH11" s="6">
-        <f>IF(S11="","",IF(OR(I11=0,V11="IGEN",W11="IGEN"),0,IF(AND(K11&lt;&gt;"IGEN",L11="IGEN",U11="NEM"),0,S11)))</f>
+        <f>IF(S11="","",IF(OR(I11=0,V11="IGEN",W11="IGEN"),0,IF(AND(K11&lt;&gt;"IGEN",L11="IGEN",U11="NEM"),0,IF(AND(H11="GYES",E11&lt;1998),0,S11))))</f>
         <v/>
       </c>
       <c r="AI11" s="6">
@@ -13239,7 +13239,7 @@
         <v/>
       </c>
       <c r="AH12" s="6">
-        <f>IF(S12="","",IF(OR(I12=0,V12="IGEN",W12="IGEN"),0,IF(AND(K12&lt;&gt;"IGEN",L12="IGEN",U12="NEM"),0,S12)))</f>
+        <f>IF(S12="","",IF(OR(I12=0,V12="IGEN",W12="IGEN"),0,IF(AND(K12&lt;&gt;"IGEN",L12="IGEN",U12="NEM"),0,IF(AND(H12="GYES",E12&lt;1998),0,S12))))</f>
         <v/>
       </c>
       <c r="AI12" s="6">
@@ -13359,7 +13359,7 @@
         <v/>
       </c>
       <c r="AH13" s="6">
-        <f>IF(S13="","",IF(OR(I13=0,V13="IGEN",W13="IGEN"),0,IF(AND(K13&lt;&gt;"IGEN",L13="IGEN",U13="NEM"),0,S13)))</f>
+        <f>IF(S13="","",IF(OR(I13=0,V13="IGEN",W13="IGEN"),0,IF(AND(K13&lt;&gt;"IGEN",L13="IGEN",U13="NEM"),0,IF(AND(H13="GYES",E13&lt;1998),0,S13))))</f>
         <v/>
       </c>
       <c r="AI13" s="6">
@@ -13479,7 +13479,7 @@
         <v/>
       </c>
       <c r="AH14" s="6">
-        <f>IF(S14="","",IF(OR(I14=0,V14="IGEN",W14="IGEN"),0,IF(AND(K14&lt;&gt;"IGEN",L14="IGEN",U14="NEM"),0,S14)))</f>
+        <f>IF(S14="","",IF(OR(I14=0,V14="IGEN",W14="IGEN"),0,IF(AND(K14&lt;&gt;"IGEN",L14="IGEN",U14="NEM"),0,IF(AND(H14="GYES",E14&lt;1998),0,S14))))</f>
         <v/>
       </c>
       <c r="AI14" s="6">
@@ -13599,7 +13599,7 @@
         <v/>
       </c>
       <c r="AH15" s="6">
-        <f>IF(S15="","",IF(OR(I15=0,V15="IGEN",W15="IGEN"),0,IF(AND(K15&lt;&gt;"IGEN",L15="IGEN",U15="NEM"),0,S15)))</f>
+        <f>IF(S15="","",IF(OR(I15=0,V15="IGEN",W15="IGEN"),0,IF(AND(K15&lt;&gt;"IGEN",L15="IGEN",U15="NEM"),0,IF(AND(H15="GYES",E15&lt;1998),0,S15))))</f>
         <v/>
       </c>
       <c r="AI15" s="6">
@@ -13719,7 +13719,7 @@
         <v/>
       </c>
       <c r="AH16" s="6">
-        <f>IF(S16="","",IF(OR(I16=0,V16="IGEN",W16="IGEN"),0,IF(AND(K16&lt;&gt;"IGEN",L16="IGEN",U16="NEM"),0,S16)))</f>
+        <f>IF(S16="","",IF(OR(I16=0,V16="IGEN",W16="IGEN"),0,IF(AND(K16&lt;&gt;"IGEN",L16="IGEN",U16="NEM"),0,IF(AND(H16="GYES",E16&lt;1998),0,S16))))</f>
         <v/>
       </c>
       <c r="AI16" s="6">
@@ -13839,7 +13839,7 @@
         <v/>
       </c>
       <c r="AH17" s="6">
-        <f>IF(S17="","",IF(OR(I17=0,V17="IGEN",W17="IGEN"),0,IF(AND(K17&lt;&gt;"IGEN",L17="IGEN",U17="NEM"),0,S17)))</f>
+        <f>IF(S17="","",IF(OR(I17=0,V17="IGEN",W17="IGEN"),0,IF(AND(K17&lt;&gt;"IGEN",L17="IGEN",U17="NEM"),0,IF(AND(H17="GYES",E17&lt;1998),0,S17))))</f>
         <v/>
       </c>
       <c r="AI17" s="6">
@@ -13959,7 +13959,7 @@
         <v/>
       </c>
       <c r="AH18" s="6">
-        <f>IF(S18="","",IF(OR(I18=0,V18="IGEN",W18="IGEN"),0,IF(AND(K18&lt;&gt;"IGEN",L18="IGEN",U18="NEM"),0,S18)))</f>
+        <f>IF(S18="","",IF(OR(I18=0,V18="IGEN",W18="IGEN"),0,IF(AND(K18&lt;&gt;"IGEN",L18="IGEN",U18="NEM"),0,IF(AND(H18="GYES",E18&lt;1998),0,S18))))</f>
         <v/>
       </c>
       <c r="AI18" s="6">
@@ -14079,7 +14079,7 @@
         <v/>
       </c>
       <c r="AH19" s="6">
-        <f>IF(S19="","",IF(OR(I19=0,V19="IGEN",W19="IGEN"),0,IF(AND(K19&lt;&gt;"IGEN",L19="IGEN",U19="NEM"),0,S19)))</f>
+        <f>IF(S19="","",IF(OR(I19=0,V19="IGEN",W19="IGEN"),0,IF(AND(K19&lt;&gt;"IGEN",L19="IGEN",U19="NEM"),0,IF(AND(H19="GYES",E19&lt;1998),0,S19))))</f>
         <v/>
       </c>
       <c r="AI19" s="6">
@@ -14199,7 +14199,7 @@
         <v/>
       </c>
       <c r="AH20" s="6">
-        <f>IF(S20="","",IF(OR(I20=0,V20="IGEN",W20="IGEN"),0,IF(AND(K20&lt;&gt;"IGEN",L20="IGEN",U20="NEM"),0,S20)))</f>
+        <f>IF(S20="","",IF(OR(I20=0,V20="IGEN",W20="IGEN"),0,IF(AND(K20&lt;&gt;"IGEN",L20="IGEN",U20="NEM"),0,IF(AND(H20="GYES",E20&lt;1998),0,S20))))</f>
         <v/>
       </c>
       <c r="AI20" s="6">
@@ -14319,7 +14319,7 @@
         <v/>
       </c>
       <c r="AH21" s="6">
-        <f>IF(S21="","",IF(OR(I21=0,V21="IGEN",W21="IGEN"),0,IF(AND(K21&lt;&gt;"IGEN",L21="IGEN",U21="NEM"),0,S21)))</f>
+        <f>IF(S21="","",IF(OR(I21=0,V21="IGEN",W21="IGEN"),0,IF(AND(K21&lt;&gt;"IGEN",L21="IGEN",U21="NEM"),0,IF(AND(H21="GYES",E21&lt;1998),0,S21))))</f>
         <v/>
       </c>
       <c r="AI21" s="6">
@@ -14439,7 +14439,7 @@
         <v/>
       </c>
       <c r="AH22" s="6">
-        <f>IF(S22="","",IF(OR(I22=0,V22="IGEN",W22="IGEN"),0,IF(AND(K22&lt;&gt;"IGEN",L22="IGEN",U22="NEM"),0,S22)))</f>
+        <f>IF(S22="","",IF(OR(I22=0,V22="IGEN",W22="IGEN"),0,IF(AND(K22&lt;&gt;"IGEN",L22="IGEN",U22="NEM"),0,IF(AND(H22="GYES",E22&lt;1998),0,S22))))</f>
         <v/>
       </c>
       <c r="AI22" s="6">
@@ -14559,7 +14559,7 @@
         <v/>
       </c>
       <c r="AH23" s="6">
-        <f>IF(S23="","",IF(OR(I23=0,V23="IGEN",W23="IGEN"),0,IF(AND(K23&lt;&gt;"IGEN",L23="IGEN",U23="NEM"),0,S23)))</f>
+        <f>IF(S23="","",IF(OR(I23=0,V23="IGEN",W23="IGEN"),0,IF(AND(K23&lt;&gt;"IGEN",L23="IGEN",U23="NEM"),0,IF(AND(H23="GYES",E23&lt;1998),0,S23))))</f>
         <v/>
       </c>
       <c r="AI23" s="6">
@@ -14679,7 +14679,7 @@
         <v/>
       </c>
       <c r="AH24" s="6">
-        <f>IF(S24="","",IF(OR(I24=0,V24="IGEN",W24="IGEN"),0,IF(AND(K24&lt;&gt;"IGEN",L24="IGEN",U24="NEM"),0,S24)))</f>
+        <f>IF(S24="","",IF(OR(I24=0,V24="IGEN",W24="IGEN"),0,IF(AND(K24&lt;&gt;"IGEN",L24="IGEN",U24="NEM"),0,IF(AND(H24="GYES",E24&lt;1998),0,S24))))</f>
         <v/>
       </c>
       <c r="AI24" s="6">
@@ -14799,7 +14799,7 @@
         <v/>
       </c>
       <c r="AH25" s="6">
-        <f>IF(S25="","",IF(OR(I25=0,V25="IGEN",W25="IGEN"),0,IF(AND(K25&lt;&gt;"IGEN",L25="IGEN",U25="NEM"),0,S25)))</f>
+        <f>IF(S25="","",IF(OR(I25=0,V25="IGEN",W25="IGEN"),0,IF(AND(K25&lt;&gt;"IGEN",L25="IGEN",U25="NEM"),0,IF(AND(H25="GYES",E25&lt;1998),0,S25))))</f>
         <v/>
       </c>
       <c r="AI25" s="6">
@@ -14919,7 +14919,7 @@
         <v/>
       </c>
       <c r="AH26" s="6">
-        <f>IF(S26="","",IF(OR(I26=0,V26="IGEN",W26="IGEN"),0,IF(AND(K26&lt;&gt;"IGEN",L26="IGEN",U26="NEM"),0,S26)))</f>
+        <f>IF(S26="","",IF(OR(I26=0,V26="IGEN",W26="IGEN"),0,IF(AND(K26&lt;&gt;"IGEN",L26="IGEN",U26="NEM"),0,IF(AND(H26="GYES",E26&lt;1998),0,S26))))</f>
         <v/>
       </c>
       <c r="AI26" s="6">
@@ -15039,7 +15039,7 @@
         <v/>
       </c>
       <c r="AH27" s="6">
-        <f>IF(S27="","",IF(OR(I27=0,V27="IGEN",W27="IGEN"),0,IF(AND(K27&lt;&gt;"IGEN",L27="IGEN",U27="NEM"),0,S27)))</f>
+        <f>IF(S27="","",IF(OR(I27=0,V27="IGEN",W27="IGEN"),0,IF(AND(K27&lt;&gt;"IGEN",L27="IGEN",U27="NEM"),0,IF(AND(H27="GYES",E27&lt;1998),0,S27))))</f>
         <v/>
       </c>
       <c r="AI27" s="6">
@@ -15159,7 +15159,7 @@
         <v/>
       </c>
       <c r="AH28" s="6">
-        <f>IF(S28="","",IF(OR(I28=0,V28="IGEN",W28="IGEN"),0,IF(AND(K28&lt;&gt;"IGEN",L28="IGEN",U28="NEM"),0,S28)))</f>
+        <f>IF(S28="","",IF(OR(I28=0,V28="IGEN",W28="IGEN"),0,IF(AND(K28&lt;&gt;"IGEN",L28="IGEN",U28="NEM"),0,IF(AND(H28="GYES",E28&lt;1998),0,S28))))</f>
         <v/>
       </c>
       <c r="AI28" s="6">
@@ -15279,7 +15279,7 @@
         <v/>
       </c>
       <c r="AH29" s="6">
-        <f>IF(S29="","",IF(OR(I29=0,V29="IGEN",W29="IGEN"),0,IF(AND(K29&lt;&gt;"IGEN",L29="IGEN",U29="NEM"),0,S29)))</f>
+        <f>IF(S29="","",IF(OR(I29=0,V29="IGEN",W29="IGEN"),0,IF(AND(K29&lt;&gt;"IGEN",L29="IGEN",U29="NEM"),0,IF(AND(H29="GYES",E29&lt;1998),0,S29))))</f>
         <v/>
       </c>
       <c r="AI29" s="6">
@@ -15399,7 +15399,7 @@
         <v/>
       </c>
       <c r="AH30" s="6">
-        <f>IF(S30="","",IF(OR(I30=0,V30="IGEN",W30="IGEN"),0,IF(AND(K30&lt;&gt;"IGEN",L30="IGEN",U30="NEM"),0,S30)))</f>
+        <f>IF(S30="","",IF(OR(I30=0,V30="IGEN",W30="IGEN"),0,IF(AND(K30&lt;&gt;"IGEN",L30="IGEN",U30="NEM"),0,IF(AND(H30="GYES",E30&lt;1998),0,S30))))</f>
         <v/>
       </c>
       <c r="AI30" s="6">
@@ -15519,7 +15519,7 @@
         <v/>
       </c>
       <c r="AH31" s="6">
-        <f>IF(S31="","",IF(OR(I31=0,V31="IGEN",W31="IGEN"),0,IF(AND(K31&lt;&gt;"IGEN",L31="IGEN",U31="NEM"),0,S31)))</f>
+        <f>IF(S31="","",IF(OR(I31=0,V31="IGEN",W31="IGEN"),0,IF(AND(K31&lt;&gt;"IGEN",L31="IGEN",U31="NEM"),0,IF(AND(H31="GYES",E31&lt;1998),0,S31))))</f>
         <v/>
       </c>
       <c r="AI31" s="6">
@@ -15639,7 +15639,7 @@
         <v/>
       </c>
       <c r="AH32" s="6">
-        <f>IF(S32="","",IF(OR(I32=0,V32="IGEN",W32="IGEN"),0,IF(AND(K32&lt;&gt;"IGEN",L32="IGEN",U32="NEM"),0,S32)))</f>
+        <f>IF(S32="","",IF(OR(I32=0,V32="IGEN",W32="IGEN"),0,IF(AND(K32&lt;&gt;"IGEN",L32="IGEN",U32="NEM"),0,IF(AND(H32="GYES",E32&lt;1998),0,S32))))</f>
         <v/>
       </c>
       <c r="AI32" s="6">
@@ -15759,7 +15759,7 @@
         <v/>
       </c>
       <c r="AH33" s="6">
-        <f>IF(S33="","",IF(OR(I33=0,V33="IGEN",W33="IGEN"),0,IF(AND(K33&lt;&gt;"IGEN",L33="IGEN",U33="NEM"),0,S33)))</f>
+        <f>IF(S33="","",IF(OR(I33=0,V33="IGEN",W33="IGEN"),0,IF(AND(K33&lt;&gt;"IGEN",L33="IGEN",U33="NEM"),0,IF(AND(H33="GYES",E33&lt;1998),0,S33))))</f>
         <v/>
       </c>
       <c r="AI33" s="6">
@@ -15879,7 +15879,7 @@
         <v/>
       </c>
       <c r="AH34" s="6">
-        <f>IF(S34="","",IF(OR(I34=0,V34="IGEN",W34="IGEN"),0,IF(AND(K34&lt;&gt;"IGEN",L34="IGEN",U34="NEM"),0,S34)))</f>
+        <f>IF(S34="","",IF(OR(I34=0,V34="IGEN",W34="IGEN"),0,IF(AND(K34&lt;&gt;"IGEN",L34="IGEN",U34="NEM"),0,IF(AND(H34="GYES",E34&lt;1998),0,S34))))</f>
         <v/>
       </c>
       <c r="AI34" s="6">
@@ -15999,7 +15999,7 @@
         <v/>
       </c>
       <c r="AH35" s="6">
-        <f>IF(S35="","",IF(OR(I35=0,V35="IGEN",W35="IGEN"),0,IF(AND(K35&lt;&gt;"IGEN",L35="IGEN",U35="NEM"),0,S35)))</f>
+        <f>IF(S35="","",IF(OR(I35=0,V35="IGEN",W35="IGEN"),0,IF(AND(K35&lt;&gt;"IGEN",L35="IGEN",U35="NEM"),0,IF(AND(H35="GYES",E35&lt;1998),0,S35))))</f>
         <v/>
       </c>
       <c r="AI35" s="6">
@@ -16119,7 +16119,7 @@
         <v/>
       </c>
       <c r="AH36" s="6">
-        <f>IF(S36="","",IF(OR(I36=0,V36="IGEN",W36="IGEN"),0,IF(AND(K36&lt;&gt;"IGEN",L36="IGEN",U36="NEM"),0,S36)))</f>
+        <f>IF(S36="","",IF(OR(I36=0,V36="IGEN",W36="IGEN"),0,IF(AND(K36&lt;&gt;"IGEN",L36="IGEN",U36="NEM"),0,IF(AND(H36="GYES",E36&lt;1998),0,S36))))</f>
         <v/>
       </c>
       <c r="AI36" s="6">
@@ -16239,7 +16239,7 @@
         <v/>
       </c>
       <c r="AH37" s="6">
-        <f>IF(S37="","",IF(OR(I37=0,V37="IGEN",W37="IGEN"),0,IF(AND(K37&lt;&gt;"IGEN",L37="IGEN",U37="NEM"),0,S37)))</f>
+        <f>IF(S37="","",IF(OR(I37=0,V37="IGEN",W37="IGEN"),0,IF(AND(K37&lt;&gt;"IGEN",L37="IGEN",U37="NEM"),0,IF(AND(H37="GYES",E37&lt;1998),0,S37))))</f>
         <v/>
       </c>
       <c r="AI37" s="6">
@@ -16359,7 +16359,7 @@
         <v/>
       </c>
       <c r="AH38" s="6">
-        <f>IF(S38="","",IF(OR(I38=0,V38="IGEN",W38="IGEN"),0,IF(AND(K38&lt;&gt;"IGEN",L38="IGEN",U38="NEM"),0,S38)))</f>
+        <f>IF(S38="","",IF(OR(I38=0,V38="IGEN",W38="IGEN"),0,IF(AND(K38&lt;&gt;"IGEN",L38="IGEN",U38="NEM"),0,IF(AND(H38="GYES",E38&lt;1998),0,S38))))</f>
         <v/>
       </c>
       <c r="AI38" s="6">
@@ -16479,7 +16479,7 @@
         <v/>
       </c>
       <c r="AH39" s="6">
-        <f>IF(S39="","",IF(OR(I39=0,V39="IGEN",W39="IGEN"),0,IF(AND(K39&lt;&gt;"IGEN",L39="IGEN",U39="NEM"),0,S39)))</f>
+        <f>IF(S39="","",IF(OR(I39=0,V39="IGEN",W39="IGEN"),0,IF(AND(K39&lt;&gt;"IGEN",L39="IGEN",U39="NEM"),0,IF(AND(H39="GYES",E39&lt;1998),0,S39))))</f>
         <v/>
       </c>
       <c r="AI39" s="6">
@@ -16599,7 +16599,7 @@
         <v/>
       </c>
       <c r="AH40" s="6">
-        <f>IF(S40="","",IF(OR(I40=0,V40="IGEN",W40="IGEN"),0,IF(AND(K40&lt;&gt;"IGEN",L40="IGEN",U40="NEM"),0,S40)))</f>
+        <f>IF(S40="","",IF(OR(I40=0,V40="IGEN",W40="IGEN"),0,IF(AND(K40&lt;&gt;"IGEN",L40="IGEN",U40="NEM"),0,IF(AND(H40="GYES",E40&lt;1998),0,S40))))</f>
         <v/>
       </c>
       <c r="AI40" s="6">
@@ -16719,7 +16719,7 @@
         <v/>
       </c>
       <c r="AH41" s="6">
-        <f>IF(S41="","",IF(OR(I41=0,V41="IGEN",W41="IGEN"),0,IF(AND(K41&lt;&gt;"IGEN",L41="IGEN",U41="NEM"),0,S41)))</f>
+        <f>IF(S41="","",IF(OR(I41=0,V41="IGEN",W41="IGEN"),0,IF(AND(K41&lt;&gt;"IGEN",L41="IGEN",U41="NEM"),0,IF(AND(H41="GYES",E41&lt;1998),0,S41))))</f>
         <v/>
       </c>
       <c r="AI41" s="6">
@@ -16839,7 +16839,7 @@
         <v/>
       </c>
       <c r="AH42" s="6">
-        <f>IF(S42="","",IF(OR(I42=0,V42="IGEN",W42="IGEN"),0,IF(AND(K42&lt;&gt;"IGEN",L42="IGEN",U42="NEM"),0,S42)))</f>
+        <f>IF(S42="","",IF(OR(I42=0,V42="IGEN",W42="IGEN"),0,IF(AND(K42&lt;&gt;"IGEN",L42="IGEN",U42="NEM"),0,IF(AND(H42="GYES",E42&lt;1998),0,S42))))</f>
         <v/>
       </c>
       <c r="AI42" s="6">
@@ -16959,7 +16959,7 @@
         <v/>
       </c>
       <c r="AH43" s="6">
-        <f>IF(S43="","",IF(OR(I43=0,V43="IGEN",W43="IGEN"),0,IF(AND(K43&lt;&gt;"IGEN",L43="IGEN",U43="NEM"),0,S43)))</f>
+        <f>IF(S43="","",IF(OR(I43=0,V43="IGEN",W43="IGEN"),0,IF(AND(K43&lt;&gt;"IGEN",L43="IGEN",U43="NEM"),0,IF(AND(H43="GYES",E43&lt;1998),0,S43))))</f>
         <v/>
       </c>
       <c r="AI43" s="6">
@@ -17079,7 +17079,7 @@
         <v/>
       </c>
       <c r="AH44" s="6">
-        <f>IF(S44="","",IF(OR(I44=0,V44="IGEN",W44="IGEN"),0,IF(AND(K44&lt;&gt;"IGEN",L44="IGEN",U44="NEM"),0,S44)))</f>
+        <f>IF(S44="","",IF(OR(I44=0,V44="IGEN",W44="IGEN"),0,IF(AND(K44&lt;&gt;"IGEN",L44="IGEN",U44="NEM"),0,IF(AND(H44="GYES",E44&lt;1998),0,S44))))</f>
         <v/>
       </c>
       <c r="AI44" s="6">
@@ -17199,7 +17199,7 @@
         <v/>
       </c>
       <c r="AH45" s="6">
-        <f>IF(S45="","",IF(OR(I45=0,V45="IGEN",W45="IGEN"),0,IF(AND(K45&lt;&gt;"IGEN",L45="IGEN",U45="NEM"),0,S45)))</f>
+        <f>IF(S45="","",IF(OR(I45=0,V45="IGEN",W45="IGEN"),0,IF(AND(K45&lt;&gt;"IGEN",L45="IGEN",U45="NEM"),0,IF(AND(H45="GYES",E45&lt;1998),0,S45))))</f>
         <v/>
       </c>
       <c r="AI45" s="6">
@@ -17319,7 +17319,7 @@
         <v/>
       </c>
       <c r="AH46" s="6">
-        <f>IF(S46="","",IF(OR(I46=0,V46="IGEN",W46="IGEN"),0,IF(AND(K46&lt;&gt;"IGEN",L46="IGEN",U46="NEM"),0,S46)))</f>
+        <f>IF(S46="","",IF(OR(I46=0,V46="IGEN",W46="IGEN"),0,IF(AND(K46&lt;&gt;"IGEN",L46="IGEN",U46="NEM"),0,IF(AND(H46="GYES",E46&lt;1998),0,S46))))</f>
         <v/>
       </c>
       <c r="AI46" s="6">
@@ -17439,7 +17439,7 @@
         <v/>
       </c>
       <c r="AH47" s="6">
-        <f>IF(S47="","",IF(OR(I47=0,V47="IGEN",W47="IGEN"),0,IF(AND(K47&lt;&gt;"IGEN",L47="IGEN",U47="NEM"),0,S47)))</f>
+        <f>IF(S47="","",IF(OR(I47=0,V47="IGEN",W47="IGEN"),0,IF(AND(K47&lt;&gt;"IGEN",L47="IGEN",U47="NEM"),0,IF(AND(H47="GYES",E47&lt;1998),0,S47))))</f>
         <v/>
       </c>
       <c r="AI47" s="6">
@@ -17559,7 +17559,7 @@
         <v/>
       </c>
       <c r="AH48" s="6">
-        <f>IF(S48="","",IF(OR(I48=0,V48="IGEN",W48="IGEN"),0,IF(AND(K48&lt;&gt;"IGEN",L48="IGEN",U48="NEM"),0,S48)))</f>
+        <f>IF(S48="","",IF(OR(I48=0,V48="IGEN",W48="IGEN"),0,IF(AND(K48&lt;&gt;"IGEN",L48="IGEN",U48="NEM"),0,IF(AND(H48="GYES",E48&lt;1998),0,S48))))</f>
         <v/>
       </c>
       <c r="AI48" s="6">
@@ -17679,7 +17679,7 @@
         <v/>
       </c>
       <c r="AH49" s="6">
-        <f>IF(S49="","",IF(OR(I49=0,V49="IGEN",W49="IGEN"),0,IF(AND(K49&lt;&gt;"IGEN",L49="IGEN",U49="NEM"),0,S49)))</f>
+        <f>IF(S49="","",IF(OR(I49=0,V49="IGEN",W49="IGEN"),0,IF(AND(K49&lt;&gt;"IGEN",L49="IGEN",U49="NEM"),0,IF(AND(H49="GYES",E49&lt;1998),0,S49))))</f>
         <v/>
       </c>
       <c r="AI49" s="6">
@@ -17799,7 +17799,7 @@
         <v/>
       </c>
       <c r="AH50" s="6">
-        <f>IF(S50="","",IF(OR(I50=0,V50="IGEN",W50="IGEN"),0,IF(AND(K50&lt;&gt;"IGEN",L50="IGEN",U50="NEM"),0,S50)))</f>
+        <f>IF(S50="","",IF(OR(I50=0,V50="IGEN",W50="IGEN"),0,IF(AND(K50&lt;&gt;"IGEN",L50="IGEN",U50="NEM"),0,IF(AND(H50="GYES",E50&lt;1998),0,S50))))</f>
         <v/>
       </c>
       <c r="AI50" s="6">
@@ -17919,7 +17919,7 @@
         <v/>
       </c>
       <c r="AH51" s="6">
-        <f>IF(S51="","",IF(OR(I51=0,V51="IGEN",W51="IGEN"),0,IF(AND(K51&lt;&gt;"IGEN",L51="IGEN",U51="NEM"),0,S51)))</f>
+        <f>IF(S51="","",IF(OR(I51=0,V51="IGEN",W51="IGEN"),0,IF(AND(K51&lt;&gt;"IGEN",L51="IGEN",U51="NEM"),0,IF(AND(H51="GYES",E51&lt;1998),0,S51))))</f>
         <v/>
       </c>
       <c r="AI51" s="6">
@@ -18039,7 +18039,7 @@
         <v/>
       </c>
       <c r="AH52" s="6">
-        <f>IF(S52="","",IF(OR(I52=0,V52="IGEN",W52="IGEN"),0,IF(AND(K52&lt;&gt;"IGEN",L52="IGEN",U52="NEM"),0,S52)))</f>
+        <f>IF(S52="","",IF(OR(I52=0,V52="IGEN",W52="IGEN"),0,IF(AND(K52&lt;&gt;"IGEN",L52="IGEN",U52="NEM"),0,IF(AND(H52="GYES",E52&lt;1998),0,S52))))</f>
         <v/>
       </c>
       <c r="AI52" s="6">
@@ -18159,7 +18159,7 @@
         <v/>
       </c>
       <c r="AH53" s="6">
-        <f>IF(S53="","",IF(OR(I53=0,V53="IGEN",W53="IGEN"),0,IF(AND(K53&lt;&gt;"IGEN",L53="IGEN",U53="NEM"),0,S53)))</f>
+        <f>IF(S53="","",IF(OR(I53=0,V53="IGEN",W53="IGEN"),0,IF(AND(K53&lt;&gt;"IGEN",L53="IGEN",U53="NEM"),0,IF(AND(H53="GYES",E53&lt;1998),0,S53))))</f>
         <v/>
       </c>
       <c r="AI53" s="6">
@@ -18279,7 +18279,7 @@
         <v/>
       </c>
       <c r="AH54" s="6">
-        <f>IF(S54="","",IF(OR(I54=0,V54="IGEN",W54="IGEN"),0,IF(AND(K54&lt;&gt;"IGEN",L54="IGEN",U54="NEM"),0,S54)))</f>
+        <f>IF(S54="","",IF(OR(I54=0,V54="IGEN",W54="IGEN"),0,IF(AND(K54&lt;&gt;"IGEN",L54="IGEN",U54="NEM"),0,IF(AND(H54="GYES",E54&lt;1998),0,S54))))</f>
         <v/>
       </c>
       <c r="AI54" s="6">
@@ -18399,7 +18399,7 @@
         <v/>
       </c>
       <c r="AH55" s="6">
-        <f>IF(S55="","",IF(OR(I55=0,V55="IGEN",W55="IGEN"),0,IF(AND(K55&lt;&gt;"IGEN",L55="IGEN",U55="NEM"),0,S55)))</f>
+        <f>IF(S55="","",IF(OR(I55=0,V55="IGEN",W55="IGEN"),0,IF(AND(K55&lt;&gt;"IGEN",L55="IGEN",U55="NEM"),0,IF(AND(H55="GYES",E55&lt;1998),0,S55))))</f>
         <v/>
       </c>
       <c r="AI55" s="6">
@@ -18519,7 +18519,7 @@
         <v/>
       </c>
       <c r="AH56" s="6">
-        <f>IF(S56="","",IF(OR(I56=0,V56="IGEN",W56="IGEN"),0,IF(AND(K56&lt;&gt;"IGEN",L56="IGEN",U56="NEM"),0,S56)))</f>
+        <f>IF(S56="","",IF(OR(I56=0,V56="IGEN",W56="IGEN"),0,IF(AND(K56&lt;&gt;"IGEN",L56="IGEN",U56="NEM"),0,IF(AND(H56="GYES",E56&lt;1998),0,S56))))</f>
         <v/>
       </c>
       <c r="AI56" s="6">
@@ -18639,7 +18639,7 @@
         <v/>
       </c>
       <c r="AH57" s="6">
-        <f>IF(S57="","",IF(OR(I57=0,V57="IGEN",W57="IGEN"),0,IF(AND(K57&lt;&gt;"IGEN",L57="IGEN",U57="NEM"),0,S57)))</f>
+        <f>IF(S57="","",IF(OR(I57=0,V57="IGEN",W57="IGEN"),0,IF(AND(K57&lt;&gt;"IGEN",L57="IGEN",U57="NEM"),0,IF(AND(H57="GYES",E57&lt;1998),0,S57))))</f>
         <v/>
       </c>
       <c r="AI57" s="6">
@@ -18759,7 +18759,7 @@
         <v/>
       </c>
       <c r="AH58" s="6">
-        <f>IF(S58="","",IF(OR(I58=0,V58="IGEN",W58="IGEN"),0,IF(AND(K58&lt;&gt;"IGEN",L58="IGEN",U58="NEM"),0,S58)))</f>
+        <f>IF(S58="","",IF(OR(I58=0,V58="IGEN",W58="IGEN"),0,IF(AND(K58&lt;&gt;"IGEN",L58="IGEN",U58="NEM"),0,IF(AND(H58="GYES",E58&lt;1998),0,S58))))</f>
         <v/>
       </c>
       <c r="AI58" s="6">
@@ -18879,7 +18879,7 @@
         <v/>
       </c>
       <c r="AH59" s="6">
-        <f>IF(S59="","",IF(OR(I59=0,V59="IGEN",W59="IGEN"),0,IF(AND(K59&lt;&gt;"IGEN",L59="IGEN",U59="NEM"),0,S59)))</f>
+        <f>IF(S59="","",IF(OR(I59=0,V59="IGEN",W59="IGEN"),0,IF(AND(K59&lt;&gt;"IGEN",L59="IGEN",U59="NEM"),0,IF(AND(H59="GYES",E59&lt;1998),0,S59))))</f>
         <v/>
       </c>
       <c r="AI59" s="6">
@@ -18999,7 +18999,7 @@
         <v/>
       </c>
       <c r="AH60" s="6">
-        <f>IF(S60="","",IF(OR(I60=0,V60="IGEN",W60="IGEN"),0,IF(AND(K60&lt;&gt;"IGEN",L60="IGEN",U60="NEM"),0,S60)))</f>
+        <f>IF(S60="","",IF(OR(I60=0,V60="IGEN",W60="IGEN"),0,IF(AND(K60&lt;&gt;"IGEN",L60="IGEN",U60="NEM"),0,IF(AND(H60="GYES",E60&lt;1998),0,S60))))</f>
         <v/>
       </c>
       <c r="AI60" s="6">
@@ -19119,7 +19119,7 @@
         <v/>
       </c>
       <c r="AH61" s="6">
-        <f>IF(S61="","",IF(OR(I61=0,V61="IGEN",W61="IGEN"),0,IF(AND(K61&lt;&gt;"IGEN",L61="IGEN",U61="NEM"),0,S61)))</f>
+        <f>IF(S61="","",IF(OR(I61=0,V61="IGEN",W61="IGEN"),0,IF(AND(K61&lt;&gt;"IGEN",L61="IGEN",U61="NEM"),0,IF(AND(H61="GYES",E61&lt;1998),0,S61))))</f>
         <v/>
       </c>
       <c r="AI61" s="6">
@@ -19239,7 +19239,7 @@
         <v/>
       </c>
       <c r="AH62" s="6">
-        <f>IF(S62="","",IF(OR(I62=0,V62="IGEN",W62="IGEN"),0,IF(AND(K62&lt;&gt;"IGEN",L62="IGEN",U62="NEM"),0,S62)))</f>
+        <f>IF(S62="","",IF(OR(I62=0,V62="IGEN",W62="IGEN"),0,IF(AND(K62&lt;&gt;"IGEN",L62="IGEN",U62="NEM"),0,IF(AND(H62="GYES",E62&lt;1998),0,S62))))</f>
         <v/>
       </c>
       <c r="AI62" s="6">
@@ -19359,7 +19359,7 @@
         <v/>
       </c>
       <c r="AH63" s="6">
-        <f>IF(S63="","",IF(OR(I63=0,V63="IGEN",W63="IGEN"),0,IF(AND(K63&lt;&gt;"IGEN",L63="IGEN",U63="NEM"),0,S63)))</f>
+        <f>IF(S63="","",IF(OR(I63=0,V63="IGEN",W63="IGEN"),0,IF(AND(K63&lt;&gt;"IGEN",L63="IGEN",U63="NEM"),0,IF(AND(H63="GYES",E63&lt;1998),0,S63))))</f>
         <v/>
       </c>
       <c r="AI63" s="6">
@@ -19479,7 +19479,7 @@
         <v/>
       </c>
       <c r="AH64" s="6">
-        <f>IF(S64="","",IF(OR(I64=0,V64="IGEN",W64="IGEN"),0,IF(AND(K64&lt;&gt;"IGEN",L64="IGEN",U64="NEM"),0,S64)))</f>
+        <f>IF(S64="","",IF(OR(I64=0,V64="IGEN",W64="IGEN"),0,IF(AND(K64&lt;&gt;"IGEN",L64="IGEN",U64="NEM"),0,IF(AND(H64="GYES",E64&lt;1998),0,S64))))</f>
         <v/>
       </c>
       <c r="AI64" s="6">
@@ -19599,7 +19599,7 @@
         <v/>
       </c>
       <c r="AH65" s="6">
-        <f>IF(S65="","",IF(OR(I65=0,V65="IGEN",W65="IGEN"),0,IF(AND(K65&lt;&gt;"IGEN",L65="IGEN",U65="NEM"),0,S65)))</f>
+        <f>IF(S65="","",IF(OR(I65=0,V65="IGEN",W65="IGEN"),0,IF(AND(K65&lt;&gt;"IGEN",L65="IGEN",U65="NEM"),0,IF(AND(H65="GYES",E65&lt;1998),0,S65))))</f>
         <v/>
       </c>
       <c r="AI65" s="6">
@@ -19719,7 +19719,7 @@
         <v/>
       </c>
       <c r="AH66" s="6">
-        <f>IF(S66="","",IF(OR(I66=0,V66="IGEN",W66="IGEN"),0,IF(AND(K66&lt;&gt;"IGEN",L66="IGEN",U66="NEM"),0,S66)))</f>
+        <f>IF(S66="","",IF(OR(I66=0,V66="IGEN",W66="IGEN"),0,IF(AND(K66&lt;&gt;"IGEN",L66="IGEN",U66="NEM"),0,IF(AND(H66="GYES",E66&lt;1998),0,S66))))</f>
         <v/>
       </c>
       <c r="AI66" s="6">
@@ -19839,7 +19839,7 @@
         <v/>
       </c>
       <c r="AH67" s="6">
-        <f>IF(S67="","",IF(OR(I67=0,V67="IGEN",W67="IGEN"),0,IF(AND(K67&lt;&gt;"IGEN",L67="IGEN",U67="NEM"),0,S67)))</f>
+        <f>IF(S67="","",IF(OR(I67=0,V67="IGEN",W67="IGEN"),0,IF(AND(K67&lt;&gt;"IGEN",L67="IGEN",U67="NEM"),0,IF(AND(H67="GYES",E67&lt;1998),0,S67))))</f>
         <v/>
       </c>
       <c r="AI67" s="6">
@@ -19959,7 +19959,7 @@
         <v/>
       </c>
       <c r="AH68" s="6">
-        <f>IF(S68="","",IF(OR(I68=0,V68="IGEN",W68="IGEN"),0,IF(AND(K68&lt;&gt;"IGEN",L68="IGEN",U68="NEM"),0,S68)))</f>
+        <f>IF(S68="","",IF(OR(I68=0,V68="IGEN",W68="IGEN"),0,IF(AND(K68&lt;&gt;"IGEN",L68="IGEN",U68="NEM"),0,IF(AND(H68="GYES",E68&lt;1998),0,S68))))</f>
         <v/>
       </c>
       <c r="AI68" s="6">
@@ -20079,7 +20079,7 @@
         <v/>
       </c>
       <c r="AH69" s="6">
-        <f>IF(S69="","",IF(OR(I69=0,V69="IGEN",W69="IGEN"),0,IF(AND(K69&lt;&gt;"IGEN",L69="IGEN",U69="NEM"),0,S69)))</f>
+        <f>IF(S69="","",IF(OR(I69=0,V69="IGEN",W69="IGEN"),0,IF(AND(K69&lt;&gt;"IGEN",L69="IGEN",U69="NEM"),0,IF(AND(H69="GYES",E69&lt;1998),0,S69))))</f>
         <v/>
       </c>
       <c r="AI69" s="6">
@@ -20199,7 +20199,7 @@
         <v/>
       </c>
       <c r="AH70" s="6">
-        <f>IF(S70="","",IF(OR(I70=0,V70="IGEN",W70="IGEN"),0,IF(AND(K70&lt;&gt;"IGEN",L70="IGEN",U70="NEM"),0,S70)))</f>
+        <f>IF(S70="","",IF(OR(I70=0,V70="IGEN",W70="IGEN"),0,IF(AND(K70&lt;&gt;"IGEN",L70="IGEN",U70="NEM"),0,IF(AND(H70="GYES",E70&lt;1998),0,S70))))</f>
         <v/>
       </c>
       <c r="AI70" s="6">
@@ -20319,7 +20319,7 @@
         <v/>
       </c>
       <c r="AH71" s="6">
-        <f>IF(S71="","",IF(OR(I71=0,V71="IGEN",W71="IGEN"),0,IF(AND(K71&lt;&gt;"IGEN",L71="IGEN",U71="NEM"),0,S71)))</f>
+        <f>IF(S71="","",IF(OR(I71=0,V71="IGEN",W71="IGEN"),0,IF(AND(K71&lt;&gt;"IGEN",L71="IGEN",U71="NEM"),0,IF(AND(H71="GYES",E71&lt;1998),0,S71))))</f>
         <v/>
       </c>
       <c r="AI71" s="6">
@@ -20439,7 +20439,7 @@
         <v/>
       </c>
       <c r="AH72" s="6">
-        <f>IF(S72="","",IF(OR(I72=0,V72="IGEN",W72="IGEN"),0,IF(AND(K72&lt;&gt;"IGEN",L72="IGEN",U72="NEM"),0,S72)))</f>
+        <f>IF(S72="","",IF(OR(I72=0,V72="IGEN",W72="IGEN"),0,IF(AND(K72&lt;&gt;"IGEN",L72="IGEN",U72="NEM"),0,IF(AND(H72="GYES",E72&lt;1998),0,S72))))</f>
         <v/>
       </c>
       <c r="AI72" s="6">
@@ -20559,7 +20559,7 @@
         <v/>
       </c>
       <c r="AH73" s="6">
-        <f>IF(S73="","",IF(OR(I73=0,V73="IGEN",W73="IGEN"),0,IF(AND(K73&lt;&gt;"IGEN",L73="IGEN",U73="NEM"),0,S73)))</f>
+        <f>IF(S73="","",IF(OR(I73=0,V73="IGEN",W73="IGEN"),0,IF(AND(K73&lt;&gt;"IGEN",L73="IGEN",U73="NEM"),0,IF(AND(H73="GYES",E73&lt;1998),0,S73))))</f>
         <v/>
       </c>
       <c r="AI73" s="6">
@@ -20679,7 +20679,7 @@
         <v/>
       </c>
       <c r="AH74" s="6">
-        <f>IF(S74="","",IF(OR(I74=0,V74="IGEN",W74="IGEN"),0,IF(AND(K74&lt;&gt;"IGEN",L74="IGEN",U74="NEM"),0,S74)))</f>
+        <f>IF(S74="","",IF(OR(I74=0,V74="IGEN",W74="IGEN"),0,IF(AND(K74&lt;&gt;"IGEN",L74="IGEN",U74="NEM"),0,IF(AND(H74="GYES",E74&lt;1998),0,S74))))</f>
         <v/>
       </c>
       <c r="AI74" s="6">
@@ -20799,7 +20799,7 @@
         <v/>
       </c>
       <c r="AH75" s="6">
-        <f>IF(S75="","",IF(OR(I75=0,V75="IGEN",W75="IGEN"),0,IF(AND(K75&lt;&gt;"IGEN",L75="IGEN",U75="NEM"),0,S75)))</f>
+        <f>IF(S75="","",IF(OR(I75=0,V75="IGEN",W75="IGEN"),0,IF(AND(K75&lt;&gt;"IGEN",L75="IGEN",U75="NEM"),0,IF(AND(H75="GYES",E75&lt;1998),0,S75))))</f>
         <v/>
       </c>
       <c r="AI75" s="6">
@@ -20919,7 +20919,7 @@
         <v/>
       </c>
       <c r="AH76" s="6">
-        <f>IF(S76="","",IF(OR(I76=0,V76="IGEN",W76="IGEN"),0,IF(AND(K76&lt;&gt;"IGEN",L76="IGEN",U76="NEM"),0,S76)))</f>
+        <f>IF(S76="","",IF(OR(I76=0,V76="IGEN",W76="IGEN"),0,IF(AND(K76&lt;&gt;"IGEN",L76="IGEN",U76="NEM"),0,IF(AND(H76="GYES",E76&lt;1998),0,S76))))</f>
         <v/>
       </c>
       <c r="AI76" s="6">
@@ -21039,7 +21039,7 @@
         <v/>
       </c>
       <c r="AH77" s="6">
-        <f>IF(S77="","",IF(OR(I77=0,V77="IGEN",W77="IGEN"),0,IF(AND(K77&lt;&gt;"IGEN",L77="IGEN",U77="NEM"),0,S77)))</f>
+        <f>IF(S77="","",IF(OR(I77=0,V77="IGEN",W77="IGEN"),0,IF(AND(K77&lt;&gt;"IGEN",L77="IGEN",U77="NEM"),0,IF(AND(H77="GYES",E77&lt;1998),0,S77))))</f>
         <v/>
       </c>
       <c r="AI77" s="6">
@@ -21159,7 +21159,7 @@
         <v/>
       </c>
       <c r="AH78" s="6">
-        <f>IF(S78="","",IF(OR(I78=0,V78="IGEN",W78="IGEN"),0,IF(AND(K78&lt;&gt;"IGEN",L78="IGEN",U78="NEM"),0,S78)))</f>
+        <f>IF(S78="","",IF(OR(I78=0,V78="IGEN",W78="IGEN"),0,IF(AND(K78&lt;&gt;"IGEN",L78="IGEN",U78="NEM"),0,IF(AND(H78="GYES",E78&lt;1998),0,S78))))</f>
         <v/>
       </c>
       <c r="AI78" s="6">
@@ -21279,7 +21279,7 @@
         <v/>
       </c>
       <c r="AH79" s="6">
-        <f>IF(S79="","",IF(OR(I79=0,V79="IGEN",W79="IGEN"),0,IF(AND(K79&lt;&gt;"IGEN",L79="IGEN",U79="NEM"),0,S79)))</f>
+        <f>IF(S79="","",IF(OR(I79=0,V79="IGEN",W79="IGEN"),0,IF(AND(K79&lt;&gt;"IGEN",L79="IGEN",U79="NEM"),0,IF(AND(H79="GYES",E79&lt;1998),0,S79))))</f>
         <v/>
       </c>
       <c r="AI79" s="6">
@@ -21399,7 +21399,7 @@
         <v/>
       </c>
       <c r="AH80" s="6">
-        <f>IF(S80="","",IF(OR(I80=0,V80="IGEN",W80="IGEN"),0,IF(AND(K80&lt;&gt;"IGEN",L80="IGEN",U80="NEM"),0,S80)))</f>
+        <f>IF(S80="","",IF(OR(I80=0,V80="IGEN",W80="IGEN"),0,IF(AND(K80&lt;&gt;"IGEN",L80="IGEN",U80="NEM"),0,IF(AND(H80="GYES",E80&lt;1998),0,S80))))</f>
         <v/>
       </c>
       <c r="AI80" s="6">
@@ -21519,7 +21519,7 @@
         <v/>
       </c>
       <c r="AH81" s="6">
-        <f>IF(S81="","",IF(OR(I81=0,V81="IGEN",W81="IGEN"),0,IF(AND(K81&lt;&gt;"IGEN",L81="IGEN",U81="NEM"),0,S81)))</f>
+        <f>IF(S81="","",IF(OR(I81=0,V81="IGEN",W81="IGEN"),0,IF(AND(K81&lt;&gt;"IGEN",L81="IGEN",U81="NEM"),0,IF(AND(H81="GYES",E81&lt;1998),0,S81))))</f>
         <v/>
       </c>
       <c r="AI81" s="6">
@@ -21639,7 +21639,7 @@
         <v/>
       </c>
       <c r="AH82" s="6">
-        <f>IF(S82="","",IF(OR(I82=0,V82="IGEN",W82="IGEN"),0,IF(AND(K82&lt;&gt;"IGEN",L82="IGEN",U82="NEM"),0,S82)))</f>
+        <f>IF(S82="","",IF(OR(I82=0,V82="IGEN",W82="IGEN"),0,IF(AND(K82&lt;&gt;"IGEN",L82="IGEN",U82="NEM"),0,IF(AND(H82="GYES",E82&lt;1998),0,S82))))</f>
         <v/>
       </c>
       <c r="AI82" s="6">
@@ -21759,7 +21759,7 @@
         <v/>
       </c>
       <c r="AH83" s="6">
-        <f>IF(S83="","",IF(OR(I83=0,V83="IGEN",W83="IGEN"),0,IF(AND(K83&lt;&gt;"IGEN",L83="IGEN",U83="NEM"),0,S83)))</f>
+        <f>IF(S83="","",IF(OR(I83=0,V83="IGEN",W83="IGEN"),0,IF(AND(K83&lt;&gt;"IGEN",L83="IGEN",U83="NEM"),0,IF(AND(H83="GYES",E83&lt;1998),0,S83))))</f>
         <v/>
       </c>
       <c r="AI83" s="6">
@@ -21879,7 +21879,7 @@
         <v/>
       </c>
       <c r="AH84" s="6">
-        <f>IF(S84="","",IF(OR(I84=0,V84="IGEN",W84="IGEN"),0,IF(AND(K84&lt;&gt;"IGEN",L84="IGEN",U84="NEM"),0,S84)))</f>
+        <f>IF(S84="","",IF(OR(I84=0,V84="IGEN",W84="IGEN"),0,IF(AND(K84&lt;&gt;"IGEN",L84="IGEN",U84="NEM"),0,IF(AND(H84="GYES",E84&lt;1998),0,S84))))</f>
         <v/>
       </c>
       <c r="AI84" s="6">
@@ -21999,7 +21999,7 @@
         <v/>
       </c>
       <c r="AH85" s="6">
-        <f>IF(S85="","",IF(OR(I85=0,V85="IGEN",W85="IGEN"),0,IF(AND(K85&lt;&gt;"IGEN",L85="IGEN",U85="NEM"),0,S85)))</f>
+        <f>IF(S85="","",IF(OR(I85=0,V85="IGEN",W85="IGEN"),0,IF(AND(K85&lt;&gt;"IGEN",L85="IGEN",U85="NEM"),0,IF(AND(H85="GYES",E85&lt;1998),0,S85))))</f>
         <v/>
       </c>
       <c r="AI85" s="6">
@@ -22119,7 +22119,7 @@
         <v/>
       </c>
       <c r="AH86" s="6">
-        <f>IF(S86="","",IF(OR(I86=0,V86="IGEN",W86="IGEN"),0,IF(AND(K86&lt;&gt;"IGEN",L86="IGEN",U86="NEM"),0,S86)))</f>
+        <f>IF(S86="","",IF(OR(I86=0,V86="IGEN",W86="IGEN"),0,IF(AND(K86&lt;&gt;"IGEN",L86="IGEN",U86="NEM"),0,IF(AND(H86="GYES",E86&lt;1998),0,S86))))</f>
         <v/>
       </c>
       <c r="AI86" s="6">
@@ -22239,7 +22239,7 @@
         <v/>
       </c>
       <c r="AH87" s="6">
-        <f>IF(S87="","",IF(OR(I87=0,V87="IGEN",W87="IGEN"),0,IF(AND(K87&lt;&gt;"IGEN",L87="IGEN",U87="NEM"),0,S87)))</f>
+        <f>IF(S87="","",IF(OR(I87=0,V87="IGEN",W87="IGEN"),0,IF(AND(K87&lt;&gt;"IGEN",L87="IGEN",U87="NEM"),0,IF(AND(H87="GYES",E87&lt;1998),0,S87))))</f>
         <v/>
       </c>
       <c r="AI87" s="6">
@@ -22359,7 +22359,7 @@
         <v/>
       </c>
       <c r="AH88" s="6">
-        <f>IF(S88="","",IF(OR(I88=0,V88="IGEN",W88="IGEN"),0,IF(AND(K88&lt;&gt;"IGEN",L88="IGEN",U88="NEM"),0,S88)))</f>
+        <f>IF(S88="","",IF(OR(I88=0,V88="IGEN",W88="IGEN"),0,IF(AND(K88&lt;&gt;"IGEN",L88="IGEN",U88="NEM"),0,IF(AND(H88="GYES",E88&lt;1998),0,S88))))</f>
         <v/>
       </c>
       <c r="AI88" s="6">
@@ -22479,7 +22479,7 @@
         <v/>
       </c>
       <c r="AH89" s="6">
-        <f>IF(S89="","",IF(OR(I89=0,V89="IGEN",W89="IGEN"),0,IF(AND(K89&lt;&gt;"IGEN",L89="IGEN",U89="NEM"),0,S89)))</f>
+        <f>IF(S89="","",IF(OR(I89=0,V89="IGEN",W89="IGEN"),0,IF(AND(K89&lt;&gt;"IGEN",L89="IGEN",U89="NEM"),0,IF(AND(H89="GYES",E89&lt;1998),0,S89))))</f>
         <v/>
       </c>
       <c r="AI89" s="6">
@@ -22599,7 +22599,7 @@
         <v/>
       </c>
       <c r="AH90" s="6">
-        <f>IF(S90="","",IF(OR(I90=0,V90="IGEN",W90="IGEN"),0,IF(AND(K90&lt;&gt;"IGEN",L90="IGEN",U90="NEM"),0,S90)))</f>
+        <f>IF(S90="","",IF(OR(I90=0,V90="IGEN",W90="IGEN"),0,IF(AND(K90&lt;&gt;"IGEN",L90="IGEN",U90="NEM"),0,IF(AND(H90="GYES",E90&lt;1998),0,S90))))</f>
         <v/>
       </c>
       <c r="AI90" s="6">
@@ -22719,7 +22719,7 @@
         <v/>
       </c>
       <c r="AH91" s="6">
-        <f>IF(S91="","",IF(OR(I91=0,V91="IGEN",W91="IGEN"),0,IF(AND(K91&lt;&gt;"IGEN",L91="IGEN",U91="NEM"),0,S91)))</f>
+        <f>IF(S91="","",IF(OR(I91=0,V91="IGEN",W91="IGEN"),0,IF(AND(K91&lt;&gt;"IGEN",L91="IGEN",U91="NEM"),0,IF(AND(H91="GYES",E91&lt;1998),0,S91))))</f>
         <v/>
       </c>
       <c r="AI91" s="6">
@@ -22839,7 +22839,7 @@
         <v/>
       </c>
       <c r="AH92" s="6">
-        <f>IF(S92="","",IF(OR(I92=0,V92="IGEN",W92="IGEN"),0,IF(AND(K92&lt;&gt;"IGEN",L92="IGEN",U92="NEM"),0,S92)))</f>
+        <f>IF(S92="","",IF(OR(I92=0,V92="IGEN",W92="IGEN"),0,IF(AND(K92&lt;&gt;"IGEN",L92="IGEN",U92="NEM"),0,IF(AND(H92="GYES",E92&lt;1998),0,S92))))</f>
         <v/>
       </c>
       <c r="AI92" s="6">
@@ -22959,7 +22959,7 @@
         <v/>
       </c>
       <c r="AH93" s="6">
-        <f>IF(S93="","",IF(OR(I93=0,V93="IGEN",W93="IGEN"),0,IF(AND(K93&lt;&gt;"IGEN",L93="IGEN",U93="NEM"),0,S93)))</f>
+        <f>IF(S93="","",IF(OR(I93=0,V93="IGEN",W93="IGEN"),0,IF(AND(K93&lt;&gt;"IGEN",L93="IGEN",U93="NEM"),0,IF(AND(H93="GYES",E93&lt;1998),0,S93))))</f>
         <v/>
       </c>
       <c r="AI93" s="6">
@@ -23079,7 +23079,7 @@
         <v/>
       </c>
       <c r="AH94" s="6">
-        <f>IF(S94="","",IF(OR(I94=0,V94="IGEN",W94="IGEN"),0,IF(AND(K94&lt;&gt;"IGEN",L94="IGEN",U94="NEM"),0,S94)))</f>
+        <f>IF(S94="","",IF(OR(I94=0,V94="IGEN",W94="IGEN"),0,IF(AND(K94&lt;&gt;"IGEN",L94="IGEN",U94="NEM"),0,IF(AND(H94="GYES",E94&lt;1998),0,S94))))</f>
         <v/>
       </c>
       <c r="AI94" s="6">
@@ -23199,7 +23199,7 @@
         <v/>
       </c>
       <c r="AH95" s="6">
-        <f>IF(S95="","",IF(OR(I95=0,V95="IGEN",W95="IGEN"),0,IF(AND(K95&lt;&gt;"IGEN",L95="IGEN",U95="NEM"),0,S95)))</f>
+        <f>IF(S95="","",IF(OR(I95=0,V95="IGEN",W95="IGEN"),0,IF(AND(K95&lt;&gt;"IGEN",L95="IGEN",U95="NEM"),0,IF(AND(H95="GYES",E95&lt;1998),0,S95))))</f>
         <v/>
       </c>
       <c r="AI95" s="6">
@@ -23319,7 +23319,7 @@
         <v/>
       </c>
       <c r="AH96" s="6">
-        <f>IF(S96="","",IF(OR(I96=0,V96="IGEN",W96="IGEN"),0,IF(AND(K96&lt;&gt;"IGEN",L96="IGEN",U96="NEM"),0,S96)))</f>
+        <f>IF(S96="","",IF(OR(I96=0,V96="IGEN",W96="IGEN"),0,IF(AND(K96&lt;&gt;"IGEN",L96="IGEN",U96="NEM"),0,IF(AND(H96="GYES",E96&lt;1998),0,S96))))</f>
         <v/>
       </c>
       <c r="AI96" s="6">
@@ -23439,7 +23439,7 @@
         <v/>
       </c>
       <c r="AH97" s="6">
-        <f>IF(S97="","",IF(OR(I97=0,V97="IGEN",W97="IGEN"),0,IF(AND(K97&lt;&gt;"IGEN",L97="IGEN",U97="NEM"),0,S97)))</f>
+        <f>IF(S97="","",IF(OR(I97=0,V97="IGEN",W97="IGEN"),0,IF(AND(K97&lt;&gt;"IGEN",L97="IGEN",U97="NEM"),0,IF(AND(H97="GYES",E97&lt;1998),0,S97))))</f>
         <v/>
       </c>
       <c r="AI97" s="6">
@@ -23559,7 +23559,7 @@
         <v/>
       </c>
       <c r="AH98" s="6">
-        <f>IF(S98="","",IF(OR(I98=0,V98="IGEN",W98="IGEN"),0,IF(AND(K98&lt;&gt;"IGEN",L98="IGEN",U98="NEM"),0,S98)))</f>
+        <f>IF(S98="","",IF(OR(I98=0,V98="IGEN",W98="IGEN"),0,IF(AND(K98&lt;&gt;"IGEN",L98="IGEN",U98="NEM"),0,IF(AND(H98="GYES",E98&lt;1998),0,S98))))</f>
         <v/>
       </c>
       <c r="AI98" s="6">
@@ -23679,7 +23679,7 @@
         <v/>
       </c>
       <c r="AH99" s="6">
-        <f>IF(S99="","",IF(OR(I99=0,V99="IGEN",W99="IGEN"),0,IF(AND(K99&lt;&gt;"IGEN",L99="IGEN",U99="NEM"),0,S99)))</f>
+        <f>IF(S99="","",IF(OR(I99=0,V99="IGEN",W99="IGEN"),0,IF(AND(K99&lt;&gt;"IGEN",L99="IGEN",U99="NEM"),0,IF(AND(H99="GYES",E99&lt;1998),0,S99))))</f>
         <v/>
       </c>
       <c r="AI99" s="6">
@@ -23799,7 +23799,7 @@
         <v/>
       </c>
       <c r="AH100" s="6">
-        <f>IF(S100="","",IF(OR(I100=0,V100="IGEN",W100="IGEN"),0,IF(AND(K100&lt;&gt;"IGEN",L100="IGEN",U100="NEM"),0,S100)))</f>
+        <f>IF(S100="","",IF(OR(I100=0,V100="IGEN",W100="IGEN"),0,IF(AND(K100&lt;&gt;"IGEN",L100="IGEN",U100="NEM"),0,IF(AND(H100="GYES",E100&lt;1998),0,S100))))</f>
         <v/>
       </c>
       <c r="AI100" s="6">
@@ -23919,7 +23919,7 @@
         <v/>
       </c>
       <c r="AH101" s="6">
-        <f>IF(S101="","",IF(OR(I101=0,V101="IGEN",W101="IGEN"),0,IF(AND(K101&lt;&gt;"IGEN",L101="IGEN",U101="NEM"),0,S101)))</f>
+        <f>IF(S101="","",IF(OR(I101=0,V101="IGEN",W101="IGEN"),0,IF(AND(K101&lt;&gt;"IGEN",L101="IGEN",U101="NEM"),0,IF(AND(H101="GYES",E101&lt;1998),0,S101))))</f>
         <v/>
       </c>
       <c r="AI101" s="6">
@@ -24039,7 +24039,7 @@
         <v/>
       </c>
       <c r="AH102" s="6">
-        <f>IF(S102="","",IF(OR(I102=0,V102="IGEN",W102="IGEN"),0,IF(AND(K102&lt;&gt;"IGEN",L102="IGEN",U102="NEM"),0,S102)))</f>
+        <f>IF(S102="","",IF(OR(I102=0,V102="IGEN",W102="IGEN"),0,IF(AND(K102&lt;&gt;"IGEN",L102="IGEN",U102="NEM"),0,IF(AND(H102="GYES",E102&lt;1998),0,S102))))</f>
         <v/>
       </c>
       <c r="AI102" s="6">
@@ -24159,7 +24159,7 @@
         <v/>
       </c>
       <c r="AH103" s="6">
-        <f>IF(S103="","",IF(OR(I103=0,V103="IGEN",W103="IGEN"),0,IF(AND(K103&lt;&gt;"IGEN",L103="IGEN",U103="NEM"),0,S103)))</f>
+        <f>IF(S103="","",IF(OR(I103=0,V103="IGEN",W103="IGEN"),0,IF(AND(K103&lt;&gt;"IGEN",L103="IGEN",U103="NEM"),0,IF(AND(H103="GYES",E103&lt;1998),0,S103))))</f>
         <v/>
       </c>
       <c r="AI103" s="6">
@@ -24279,7 +24279,7 @@
         <v/>
       </c>
       <c r="AH104" s="6">
-        <f>IF(S104="","",IF(OR(I104=0,V104="IGEN",W104="IGEN"),0,IF(AND(K104&lt;&gt;"IGEN",L104="IGEN",U104="NEM"),0,S104)))</f>
+        <f>IF(S104="","",IF(OR(I104=0,V104="IGEN",W104="IGEN"),0,IF(AND(K104&lt;&gt;"IGEN",L104="IGEN",U104="NEM"),0,IF(AND(H104="GYES",E104&lt;1998),0,S104))))</f>
         <v/>
       </c>
       <c r="AI104" s="6">
@@ -24399,7 +24399,7 @@
         <v/>
       </c>
       <c r="AH105" s="6">
-        <f>IF(S105="","",IF(OR(I105=0,V105="IGEN",W105="IGEN"),0,IF(AND(K105&lt;&gt;"IGEN",L105="IGEN",U105="NEM"),0,S105)))</f>
+        <f>IF(S105="","",IF(OR(I105=0,V105="IGEN",W105="IGEN"),0,IF(AND(K105&lt;&gt;"IGEN",L105="IGEN",U105="NEM"),0,IF(AND(H105="GYES",E105&lt;1998),0,S105))))</f>
         <v/>
       </c>
       <c r="AI105" s="6">
@@ -24519,7 +24519,7 @@
         <v/>
       </c>
       <c r="AH106" s="6">
-        <f>IF(S106="","",IF(OR(I106=0,V106="IGEN",W106="IGEN"),0,IF(AND(K106&lt;&gt;"IGEN",L106="IGEN",U106="NEM"),0,S106)))</f>
+        <f>IF(S106="","",IF(OR(I106=0,V106="IGEN",W106="IGEN"),0,IF(AND(K106&lt;&gt;"IGEN",L106="IGEN",U106="NEM"),0,IF(AND(H106="GYES",E106&lt;1998),0,S106))))</f>
         <v/>
       </c>
       <c r="AI106" s="6">
@@ -24639,7 +24639,7 @@
         <v/>
       </c>
       <c r="AH107" s="6">
-        <f>IF(S107="","",IF(OR(I107=0,V107="IGEN",W107="IGEN"),0,IF(AND(K107&lt;&gt;"IGEN",L107="IGEN",U107="NEM"),0,S107)))</f>
+        <f>IF(S107="","",IF(OR(I107=0,V107="IGEN",W107="IGEN"),0,IF(AND(K107&lt;&gt;"IGEN",L107="IGEN",U107="NEM"),0,IF(AND(H107="GYES",E107&lt;1998),0,S107))))</f>
         <v/>
       </c>
       <c r="AI107" s="6">
@@ -24759,7 +24759,7 @@
         <v/>
       </c>
       <c r="AH108" s="6">
-        <f>IF(S108="","",IF(OR(I108=0,V108="IGEN",W108="IGEN"),0,IF(AND(K108&lt;&gt;"IGEN",L108="IGEN",U108="NEM"),0,S108)))</f>
+        <f>IF(S108="","",IF(OR(I108=0,V108="IGEN",W108="IGEN"),0,IF(AND(K108&lt;&gt;"IGEN",L108="IGEN",U108="NEM"),0,IF(AND(H108="GYES",E108&lt;1998),0,S108))))</f>
         <v/>
       </c>
       <c r="AI108" s="6">
@@ -24879,7 +24879,7 @@
         <v/>
       </c>
       <c r="AH109" s="6">
-        <f>IF(S109="","",IF(OR(I109=0,V109="IGEN",W109="IGEN"),0,IF(AND(K109&lt;&gt;"IGEN",L109="IGEN",U109="NEM"),0,S109)))</f>
+        <f>IF(S109="","",IF(OR(I109=0,V109="IGEN",W109="IGEN"),0,IF(AND(K109&lt;&gt;"IGEN",L109="IGEN",U109="NEM"),0,IF(AND(H109="GYES",E109&lt;1998),0,S109))))</f>
         <v/>
       </c>
       <c r="AI109" s="6">
@@ -24999,7 +24999,7 @@
         <v/>
       </c>
       <c r="AH110" s="6">
-        <f>IF(S110="","",IF(OR(I110=0,V110="IGEN",W110="IGEN"),0,IF(AND(K110&lt;&gt;"IGEN",L110="IGEN",U110="NEM"),0,S110)))</f>
+        <f>IF(S110="","",IF(OR(I110=0,V110="IGEN",W110="IGEN"),0,IF(AND(K110&lt;&gt;"IGEN",L110="IGEN",U110="NEM"),0,IF(AND(H110="GYES",E110&lt;1998),0,S110))))</f>
         <v/>
       </c>
       <c r="AI110" s="6">
@@ -25119,7 +25119,7 @@
         <v/>
       </c>
       <c r="AH111" s="6">
-        <f>IF(S111="","",IF(OR(I111=0,V111="IGEN",W111="IGEN"),0,IF(AND(K111&lt;&gt;"IGEN",L111="IGEN",U111="NEM"),0,S111)))</f>
+        <f>IF(S111="","",IF(OR(I111=0,V111="IGEN",W111="IGEN"),0,IF(AND(K111&lt;&gt;"IGEN",L111="IGEN",U111="NEM"),0,IF(AND(H111="GYES",E111&lt;1998),0,S111))))</f>
         <v/>
       </c>
       <c r="AI111" s="6">
@@ -25239,7 +25239,7 @@
         <v/>
       </c>
       <c r="AH112" s="6">
-        <f>IF(S112="","",IF(OR(I112=0,V112="IGEN",W112="IGEN"),0,IF(AND(K112&lt;&gt;"IGEN",L112="IGEN",U112="NEM"),0,S112)))</f>
+        <f>IF(S112="","",IF(OR(I112=0,V112="IGEN",W112="IGEN"),0,IF(AND(K112&lt;&gt;"IGEN",L112="IGEN",U112="NEM"),0,IF(AND(H112="GYES",E112&lt;1998),0,S112))))</f>
         <v/>
       </c>
       <c r="AI112" s="6">
@@ -25359,7 +25359,7 @@
         <v/>
       </c>
       <c r="AH113" s="6">
-        <f>IF(S113="","",IF(OR(I113=0,V113="IGEN",W113="IGEN"),0,IF(AND(K113&lt;&gt;"IGEN",L113="IGEN",U113="NEM"),0,S113)))</f>
+        <f>IF(S113="","",IF(OR(I113=0,V113="IGEN",W113="IGEN"),0,IF(AND(K113&lt;&gt;"IGEN",L113="IGEN",U113="NEM"),0,IF(AND(H113="GYES",E113&lt;1998),0,S113))))</f>
         <v/>
       </c>
       <c r="AI113" s="6">
@@ -25479,7 +25479,7 @@
         <v/>
       </c>
       <c r="AH114" s="6">
-        <f>IF(S114="","",IF(OR(I114=0,V114="IGEN",W114="IGEN"),0,IF(AND(K114&lt;&gt;"IGEN",L114="IGEN",U114="NEM"),0,S114)))</f>
+        <f>IF(S114="","",IF(OR(I114=0,V114="IGEN",W114="IGEN"),0,IF(AND(K114&lt;&gt;"IGEN",L114="IGEN",U114="NEM"),0,IF(AND(H114="GYES",E114&lt;1998),0,S114))))</f>
         <v/>
       </c>
       <c r="AI114" s="6">
@@ -25599,7 +25599,7 @@
         <v/>
       </c>
       <c r="AH115" s="6">
-        <f>IF(S115="","",IF(OR(I115=0,V115="IGEN",W115="IGEN"),0,IF(AND(K115&lt;&gt;"IGEN",L115="IGEN",U115="NEM"),0,S115)))</f>
+        <f>IF(S115="","",IF(OR(I115=0,V115="IGEN",W115="IGEN"),0,IF(AND(K115&lt;&gt;"IGEN",L115="IGEN",U115="NEM"),0,IF(AND(H115="GYES",E115&lt;1998),0,S115))))</f>
         <v/>
       </c>
       <c r="AI115" s="6">
@@ -25719,7 +25719,7 @@
         <v/>
       </c>
       <c r="AH116" s="6">
-        <f>IF(S116="","",IF(OR(I116=0,V116="IGEN",W116="IGEN"),0,IF(AND(K116&lt;&gt;"IGEN",L116="IGEN",U116="NEM"),0,S116)))</f>
+        <f>IF(S116="","",IF(OR(I116=0,V116="IGEN",W116="IGEN"),0,IF(AND(K116&lt;&gt;"IGEN",L116="IGEN",U116="NEM"),0,IF(AND(H116="GYES",E116&lt;1998),0,S116))))</f>
         <v/>
       </c>
       <c r="AI116" s="6">
@@ -25839,7 +25839,7 @@
         <v/>
       </c>
       <c r="AH117" s="6">
-        <f>IF(S117="","",IF(OR(I117=0,V117="IGEN",W117="IGEN"),0,IF(AND(K117&lt;&gt;"IGEN",L117="IGEN",U117="NEM"),0,S117)))</f>
+        <f>IF(S117="","",IF(OR(I117=0,V117="IGEN",W117="IGEN"),0,IF(AND(K117&lt;&gt;"IGEN",L117="IGEN",U117="NEM"),0,IF(AND(H117="GYES",E117&lt;1998),0,S117))))</f>
         <v/>
       </c>
       <c r="AI117" s="6">
@@ -25959,7 +25959,7 @@
         <v/>
       </c>
       <c r="AH118" s="6">
-        <f>IF(S118="","",IF(OR(I118=0,V118="IGEN",W118="IGEN"),0,IF(AND(K118&lt;&gt;"IGEN",L118="IGEN",U118="NEM"),0,S118)))</f>
+        <f>IF(S118="","",IF(OR(I118=0,V118="IGEN",W118="IGEN"),0,IF(AND(K118&lt;&gt;"IGEN",L118="IGEN",U118="NEM"),0,IF(AND(H118="GYES",E118&lt;1998),0,S118))))</f>
         <v/>
       </c>
       <c r="AI118" s="6">
@@ -26079,7 +26079,7 @@
         <v/>
       </c>
       <c r="AH119" s="6">
-        <f>IF(S119="","",IF(OR(I119=0,V119="IGEN",W119="IGEN"),0,IF(AND(K119&lt;&gt;"IGEN",L119="IGEN",U119="NEM"),0,S119)))</f>
+        <f>IF(S119="","",IF(OR(I119=0,V119="IGEN",W119="IGEN"),0,IF(AND(K119&lt;&gt;"IGEN",L119="IGEN",U119="NEM"),0,IF(AND(H119="GYES",E119&lt;1998),0,S119))))</f>
         <v/>
       </c>
       <c r="AI119" s="6">
@@ -26199,7 +26199,7 @@
         <v/>
       </c>
       <c r="AH120" s="6">
-        <f>IF(S120="","",IF(OR(I120=0,V120="IGEN",W120="IGEN"),0,IF(AND(K120&lt;&gt;"IGEN",L120="IGEN",U120="NEM"),0,S120)))</f>
+        <f>IF(S120="","",IF(OR(I120=0,V120="IGEN",W120="IGEN"),0,IF(AND(K120&lt;&gt;"IGEN",L120="IGEN",U120="NEM"),0,IF(AND(H120="GYES",E120&lt;1998),0,S120))))</f>
         <v/>
       </c>
       <c r="AI120" s="6">
@@ -26319,7 +26319,7 @@
         <v/>
       </c>
       <c r="AH121" s="6">
-        <f>IF(S121="","",IF(OR(I121=0,V121="IGEN",W121="IGEN"),0,IF(AND(K121&lt;&gt;"IGEN",L121="IGEN",U121="NEM"),0,S121)))</f>
+        <f>IF(S121="","",IF(OR(I121=0,V121="IGEN",W121="IGEN"),0,IF(AND(K121&lt;&gt;"IGEN",L121="IGEN",U121="NEM"),0,IF(AND(H121="GYES",E121&lt;1998),0,S121))))</f>
         <v/>
       </c>
       <c r="AI121" s="6">
@@ -26439,7 +26439,7 @@
         <v/>
       </c>
       <c r="AH122" s="6">
-        <f>IF(S122="","",IF(OR(I122=0,V122="IGEN",W122="IGEN"),0,IF(AND(K122&lt;&gt;"IGEN",L122="IGEN",U122="NEM"),0,S122)))</f>
+        <f>IF(S122="","",IF(OR(I122=0,V122="IGEN",W122="IGEN"),0,IF(AND(K122&lt;&gt;"IGEN",L122="IGEN",U122="NEM"),0,IF(AND(H122="GYES",E122&lt;1998),0,S122))))</f>
         <v/>
       </c>
       <c r="AI122" s="6">
@@ -26559,7 +26559,7 @@
         <v/>
       </c>
       <c r="AH123" s="6">
-        <f>IF(S123="","",IF(OR(I123=0,V123="IGEN",W123="IGEN"),0,IF(AND(K123&lt;&gt;"IGEN",L123="IGEN",U123="NEM"),0,S123)))</f>
+        <f>IF(S123="","",IF(OR(I123=0,V123="IGEN",W123="IGEN"),0,IF(AND(K123&lt;&gt;"IGEN",L123="IGEN",U123="NEM"),0,IF(AND(H123="GYES",E123&lt;1998),0,S123))))</f>
         <v/>
       </c>
       <c r="AI123" s="6">
@@ -26679,7 +26679,7 @@
         <v/>
       </c>
       <c r="AH124" s="6">
-        <f>IF(S124="","",IF(OR(I124=0,V124="IGEN",W124="IGEN"),0,IF(AND(K124&lt;&gt;"IGEN",L124="IGEN",U124="NEM"),0,S124)))</f>
+        <f>IF(S124="","",IF(OR(I124=0,V124="IGEN",W124="IGEN"),0,IF(AND(K124&lt;&gt;"IGEN",L124="IGEN",U124="NEM"),0,IF(AND(H124="GYES",E124&lt;1998),0,S124))))</f>
         <v/>
       </c>
       <c r="AI124" s="6">
@@ -26799,7 +26799,7 @@
         <v/>
       </c>
       <c r="AH125" s="6">
-        <f>IF(S125="","",IF(OR(I125=0,V125="IGEN",W125="IGEN"),0,IF(AND(K125&lt;&gt;"IGEN",L125="IGEN",U125="NEM"),0,S125)))</f>
+        <f>IF(S125="","",IF(OR(I125=0,V125="IGEN",W125="IGEN"),0,IF(AND(K125&lt;&gt;"IGEN",L125="IGEN",U125="NEM"),0,IF(AND(H125="GYES",E125&lt;1998),0,S125))))</f>
         <v/>
       </c>
       <c r="AI125" s="6">
@@ -26919,7 +26919,7 @@
         <v/>
       </c>
       <c r="AH126" s="6">
-        <f>IF(S126="","",IF(OR(I126=0,V126="IGEN",W126="IGEN"),0,IF(AND(K126&lt;&gt;"IGEN",L126="IGEN",U126="NEM"),0,S126)))</f>
+        <f>IF(S126="","",IF(OR(I126=0,V126="IGEN",W126="IGEN"),0,IF(AND(K126&lt;&gt;"IGEN",L126="IGEN",U126="NEM"),0,IF(AND(H126="GYES",E126&lt;1998),0,S126))))</f>
         <v/>
       </c>
       <c r="AI126" s="6">
@@ -27039,7 +27039,7 @@
         <v/>
       </c>
       <c r="AH127" s="6">
-        <f>IF(S127="","",IF(OR(I127=0,V127="IGEN",W127="IGEN"),0,IF(AND(K127&lt;&gt;"IGEN",L127="IGEN",U127="NEM"),0,S127)))</f>
+        <f>IF(S127="","",IF(OR(I127=0,V127="IGEN",W127="IGEN"),0,IF(AND(K127&lt;&gt;"IGEN",L127="IGEN",U127="NEM"),0,IF(AND(H127="GYES",E127&lt;1998),0,S127))))</f>
         <v/>
       </c>
       <c r="AI127" s="6">
@@ -27159,7 +27159,7 @@
         <v/>
       </c>
       <c r="AH128" s="6">
-        <f>IF(S128="","",IF(OR(I128=0,V128="IGEN",W128="IGEN"),0,IF(AND(K128&lt;&gt;"IGEN",L128="IGEN",U128="NEM"),0,S128)))</f>
+        <f>IF(S128="","",IF(OR(I128=0,V128="IGEN",W128="IGEN"),0,IF(AND(K128&lt;&gt;"IGEN",L128="IGEN",U128="NEM"),0,IF(AND(H128="GYES",E128&lt;1998),0,S128))))</f>
         <v/>
       </c>
       <c r="AI128" s="6">
@@ -27279,7 +27279,7 @@
         <v/>
       </c>
       <c r="AH129" s="6">
-        <f>IF(S129="","",IF(OR(I129=0,V129="IGEN",W129="IGEN"),0,IF(AND(K129&lt;&gt;"IGEN",L129="IGEN",U129="NEM"),0,S129)))</f>
+        <f>IF(S129="","",IF(OR(I129=0,V129="IGEN",W129="IGEN"),0,IF(AND(K129&lt;&gt;"IGEN",L129="IGEN",U129="NEM"),0,IF(AND(H129="GYES",E129&lt;1998),0,S129))))</f>
         <v/>
       </c>
       <c r="AI129" s="6">
@@ -27399,7 +27399,7 @@
         <v/>
       </c>
       <c r="AH130" s="6">
-        <f>IF(S130="","",IF(OR(I130=0,V130="IGEN",W130="IGEN"),0,IF(AND(K130&lt;&gt;"IGEN",L130="IGEN",U130="NEM"),0,S130)))</f>
+        <f>IF(S130="","",IF(OR(I130=0,V130="IGEN",W130="IGEN"),0,IF(AND(K130&lt;&gt;"IGEN",L130="IGEN",U130="NEM"),0,IF(AND(H130="GYES",E130&lt;1998),0,S130))))</f>
         <v/>
       </c>
       <c r="AI130" s="6">
@@ -27519,7 +27519,7 @@
         <v/>
       </c>
       <c r="AH131" s="6">
-        <f>IF(S131="","",IF(OR(I131=0,V131="IGEN",W131="IGEN"),0,IF(AND(K131&lt;&gt;"IGEN",L131="IGEN",U131="NEM"),0,S131)))</f>
+        <f>IF(S131="","",IF(OR(I131=0,V131="IGEN",W131="IGEN"),0,IF(AND(K131&lt;&gt;"IGEN",L131="IGEN",U131="NEM"),0,IF(AND(H131="GYES",E131&lt;1998),0,S131))))</f>
         <v/>
       </c>
       <c r="AI131" s="6">
@@ -27639,7 +27639,7 @@
         <v/>
       </c>
       <c r="AH132" s="6">
-        <f>IF(S132="","",IF(OR(I132=0,V132="IGEN",W132="IGEN"),0,IF(AND(K132&lt;&gt;"IGEN",L132="IGEN",U132="NEM"),0,S132)))</f>
+        <f>IF(S132="","",IF(OR(I132=0,V132="IGEN",W132="IGEN"),0,IF(AND(K132&lt;&gt;"IGEN",L132="IGEN",U132="NEM"),0,IF(AND(H132="GYES",E132&lt;1998),0,S132))))</f>
         <v/>
       </c>
       <c r="AI132" s="6">
@@ -27759,7 +27759,7 @@
         <v/>
       </c>
       <c r="AH133" s="6">
-        <f>IF(S133="","",IF(OR(I133=0,V133="IGEN",W133="IGEN"),0,IF(AND(K133&lt;&gt;"IGEN",L133="IGEN",U133="NEM"),0,S133)))</f>
+        <f>IF(S133="","",IF(OR(I133=0,V133="IGEN",W133="IGEN"),0,IF(AND(K133&lt;&gt;"IGEN",L133="IGEN",U133="NEM"),0,IF(AND(H133="GYES",E133&lt;1998),0,S133))))</f>
         <v/>
       </c>
       <c r="AI133" s="6">
@@ -27879,7 +27879,7 @@
         <v/>
       </c>
       <c r="AH134" s="6">
-        <f>IF(S134="","",IF(OR(I134=0,V134="IGEN",W134="IGEN"),0,IF(AND(K134&lt;&gt;"IGEN",L134="IGEN",U134="NEM"),0,S134)))</f>
+        <f>IF(S134="","",IF(OR(I134=0,V134="IGEN",W134="IGEN"),0,IF(AND(K134&lt;&gt;"IGEN",L134="IGEN",U134="NEM"),0,IF(AND(H134="GYES",E134&lt;1998),0,S134))))</f>
         <v/>
       </c>
       <c r="AI134" s="6">
@@ -27999,7 +27999,7 @@
         <v/>
       </c>
       <c r="AH135" s="6">
-        <f>IF(S135="","",IF(OR(I135=0,V135="IGEN",W135="IGEN"),0,IF(AND(K135&lt;&gt;"IGEN",L135="IGEN",U135="NEM"),0,S135)))</f>
+        <f>IF(S135="","",IF(OR(I135=0,V135="IGEN",W135="IGEN"),0,IF(AND(K135&lt;&gt;"IGEN",L135="IGEN",U135="NEM"),0,IF(AND(H135="GYES",E135&lt;1998),0,S135))))</f>
         <v/>
       </c>
       <c r="AI135" s="6">
@@ -28119,7 +28119,7 @@
         <v/>
       </c>
       <c r="AH136" s="6">
-        <f>IF(S136="","",IF(OR(I136=0,V136="IGEN",W136="IGEN"),0,IF(AND(K136&lt;&gt;"IGEN",L136="IGEN",U136="NEM"),0,S136)))</f>
+        <f>IF(S136="","",IF(OR(I136=0,V136="IGEN",W136="IGEN"),0,IF(AND(K136&lt;&gt;"IGEN",L136="IGEN",U136="NEM"),0,IF(AND(H136="GYES",E136&lt;1998),0,S136))))</f>
         <v/>
       </c>
       <c r="AI136" s="6">
@@ -28239,7 +28239,7 @@
         <v/>
       </c>
       <c r="AH137" s="6">
-        <f>IF(S137="","",IF(OR(I137=0,V137="IGEN",W137="IGEN"),0,IF(AND(K137&lt;&gt;"IGEN",L137="IGEN",U137="NEM"),0,S137)))</f>
+        <f>IF(S137="","",IF(OR(I137=0,V137="IGEN",W137="IGEN"),0,IF(AND(K137&lt;&gt;"IGEN",L137="IGEN",U137="NEM"),0,IF(AND(H137="GYES",E137&lt;1998),0,S137))))</f>
         <v/>
       </c>
       <c r="AI137" s="6">
@@ -28359,7 +28359,7 @@
         <v/>
       </c>
       <c r="AH138" s="6">
-        <f>IF(S138="","",IF(OR(I138=0,V138="IGEN",W138="IGEN"),0,IF(AND(K138&lt;&gt;"IGEN",L138="IGEN",U138="NEM"),0,S138)))</f>
+        <f>IF(S138="","",IF(OR(I138=0,V138="IGEN",W138="IGEN"),0,IF(AND(K138&lt;&gt;"IGEN",L138="IGEN",U138="NEM"),0,IF(AND(H138="GYES",E138&lt;1998),0,S138))))</f>
         <v/>
       </c>
       <c r="AI138" s="6">
@@ -28479,7 +28479,7 @@
         <v/>
       </c>
       <c r="AH139" s="6">
-        <f>IF(S139="","",IF(OR(I139=0,V139="IGEN",W139="IGEN"),0,IF(AND(K139&lt;&gt;"IGEN",L139="IGEN",U139="NEM"),0,S139)))</f>
+        <f>IF(S139="","",IF(OR(I139=0,V139="IGEN",W139="IGEN"),0,IF(AND(K139&lt;&gt;"IGEN",L139="IGEN",U139="NEM"),0,IF(AND(H139="GYES",E139&lt;1998),0,S139))))</f>
         <v/>
       </c>
       <c r="AI139" s="6">
@@ -28599,7 +28599,7 @@
         <v/>
       </c>
       <c r="AH140" s="6">
-        <f>IF(S140="","",IF(OR(I140=0,V140="IGEN",W140="IGEN"),0,IF(AND(K140&lt;&gt;"IGEN",L140="IGEN",U140="NEM"),0,S140)))</f>
+        <f>IF(S140="","",IF(OR(I140=0,V140="IGEN",W140="IGEN"),0,IF(AND(K140&lt;&gt;"IGEN",L140="IGEN",U140="NEM"),0,IF(AND(H140="GYES",E140&lt;1998),0,S140))))</f>
         <v/>
       </c>
       <c r="AI140" s="6">
@@ -28719,7 +28719,7 @@
         <v/>
       </c>
       <c r="AH141" s="6">
-        <f>IF(S141="","",IF(OR(I141=0,V141="IGEN",W141="IGEN"),0,IF(AND(K141&lt;&gt;"IGEN",L141="IGEN",U141="NEM"),0,S141)))</f>
+        <f>IF(S141="","",IF(OR(I141=0,V141="IGEN",W141="IGEN"),0,IF(AND(K141&lt;&gt;"IGEN",L141="IGEN",U141="NEM"),0,IF(AND(H141="GYES",E141&lt;1998),0,S141))))</f>
         <v/>
       </c>
       <c r="AI141" s="6">
@@ -28839,7 +28839,7 @@
         <v/>
       </c>
       <c r="AH142" s="6">
-        <f>IF(S142="","",IF(OR(I142=0,V142="IGEN",W142="IGEN"),0,IF(AND(K142&lt;&gt;"IGEN",L142="IGEN",U142="NEM"),0,S142)))</f>
+        <f>IF(S142="","",IF(OR(I142=0,V142="IGEN",W142="IGEN"),0,IF(AND(K142&lt;&gt;"IGEN",L142="IGEN",U142="NEM"),0,IF(AND(H142="GYES",E142&lt;1998),0,S142))))</f>
         <v/>
       </c>
       <c r="AI142" s="6">
@@ -28959,7 +28959,7 @@
         <v/>
       </c>
       <c r="AH143" s="6">
-        <f>IF(S143="","",IF(OR(I143=0,V143="IGEN",W143="IGEN"),0,IF(AND(K143&lt;&gt;"IGEN",L143="IGEN",U143="NEM"),0,S143)))</f>
+        <f>IF(S143="","",IF(OR(I143=0,V143="IGEN",W143="IGEN"),0,IF(AND(K143&lt;&gt;"IGEN",L143="IGEN",U143="NEM"),0,IF(AND(H143="GYES",E143&lt;1998),0,S143))))</f>
         <v/>
       </c>
       <c r="AI143" s="6">
@@ -29079,7 +29079,7 @@
         <v/>
       </c>
       <c r="AH144" s="6">
-        <f>IF(S144="","",IF(OR(I144=0,V144="IGEN",W144="IGEN"),0,IF(AND(K144&lt;&gt;"IGEN",L144="IGEN",U144="NEM"),0,S144)))</f>
+        <f>IF(S144="","",IF(OR(I144=0,V144="IGEN",W144="IGEN"),0,IF(AND(K144&lt;&gt;"IGEN",L144="IGEN",U144="NEM"),0,IF(AND(H144="GYES",E144&lt;1998),0,S144))))</f>
         <v/>
       </c>
       <c r="AI144" s="6">
@@ -29199,7 +29199,7 @@
         <v/>
       </c>
       <c r="AH145" s="6">
-        <f>IF(S145="","",IF(OR(I145=0,V145="IGEN",W145="IGEN"),0,IF(AND(K145&lt;&gt;"IGEN",L145="IGEN",U145="NEM"),0,S145)))</f>
+        <f>IF(S145="","",IF(OR(I145=0,V145="IGEN",W145="IGEN"),0,IF(AND(K145&lt;&gt;"IGEN",L145="IGEN",U145="NEM"),0,IF(AND(H145="GYES",E145&lt;1998),0,S145))))</f>
         <v/>
       </c>
       <c r="AI145" s="6">
@@ -29319,7 +29319,7 @@
         <v/>
       </c>
       <c r="AH146" s="6">
-        <f>IF(S146="","",IF(OR(I146=0,V146="IGEN",W146="IGEN"),0,IF(AND(K146&lt;&gt;"IGEN",L146="IGEN",U146="NEM"),0,S146)))</f>
+        <f>IF(S146="","",IF(OR(I146=0,V146="IGEN",W146="IGEN"),0,IF(AND(K146&lt;&gt;"IGEN",L146="IGEN",U146="NEM"),0,IF(AND(H146="GYES",E146&lt;1998),0,S146))))</f>
         <v/>
       </c>
       <c r="AI146" s="6">
@@ -29439,7 +29439,7 @@
         <v/>
       </c>
       <c r="AH147" s="6">
-        <f>IF(S147="","",IF(OR(I147=0,V147="IGEN",W147="IGEN"),0,IF(AND(K147&lt;&gt;"IGEN",L147="IGEN",U147="NEM"),0,S147)))</f>
+        <f>IF(S147="","",IF(OR(I147=0,V147="IGEN",W147="IGEN"),0,IF(AND(K147&lt;&gt;"IGEN",L147="IGEN",U147="NEM"),0,IF(AND(H147="GYES",E147&lt;1998),0,S147))))</f>
         <v/>
       </c>
       <c r="AI147" s="6">
@@ -29559,7 +29559,7 @@
         <v/>
       </c>
       <c r="AH148" s="6">
-        <f>IF(S148="","",IF(OR(I148=0,V148="IGEN",W148="IGEN"),0,IF(AND(K148&lt;&gt;"IGEN",L148="IGEN",U148="NEM"),0,S148)))</f>
+        <f>IF(S148="","",IF(OR(I148=0,V148="IGEN",W148="IGEN"),0,IF(AND(K148&lt;&gt;"IGEN",L148="IGEN",U148="NEM"),0,IF(AND(H148="GYES",E148&lt;1998),0,S148))))</f>
         <v/>
       </c>
       <c r="AI148" s="6">
@@ -29679,7 +29679,7 @@
         <v/>
       </c>
       <c r="AH149" s="6">
-        <f>IF(S149="","",IF(OR(I149=0,V149="IGEN",W149="IGEN"),0,IF(AND(K149&lt;&gt;"IGEN",L149="IGEN",U149="NEM"),0,S149)))</f>
+        <f>IF(S149="","",IF(OR(I149=0,V149="IGEN",W149="IGEN"),0,IF(AND(K149&lt;&gt;"IGEN",L149="IGEN",U149="NEM"),0,IF(AND(H149="GYES",E149&lt;1998),0,S149))))</f>
         <v/>
       </c>
       <c r="AI149" s="6">
@@ -29799,7 +29799,7 @@
         <v/>
       </c>
       <c r="AH150" s="6">
-        <f>IF(S150="","",IF(OR(I150=0,V150="IGEN",W150="IGEN"),0,IF(AND(K150&lt;&gt;"IGEN",L150="IGEN",U150="NEM"),0,S150)))</f>
+        <f>IF(S150="","",IF(OR(I150=0,V150="IGEN",W150="IGEN"),0,IF(AND(K150&lt;&gt;"IGEN",L150="IGEN",U150="NEM"),0,IF(AND(H150="GYES",E150&lt;1998),0,S150))))</f>
         <v/>
       </c>
       <c r="AI150" s="6">
@@ -29919,7 +29919,7 @@
         <v/>
       </c>
       <c r="AH151" s="6">
-        <f>IF(S151="","",IF(OR(I151=0,V151="IGEN",W151="IGEN"),0,IF(AND(K151&lt;&gt;"IGEN",L151="IGEN",U151="NEM"),0,S151)))</f>
+        <f>IF(S151="","",IF(OR(I151=0,V151="IGEN",W151="IGEN"),0,IF(AND(K151&lt;&gt;"IGEN",L151="IGEN",U151="NEM"),0,IF(AND(H151="GYES",E151&lt;1998),0,S151))))</f>
         <v/>
       </c>
       <c r="AI151" s="6">
@@ -30039,7 +30039,7 @@
         <v/>
       </c>
       <c r="AH152" s="6">
-        <f>IF(S152="","",IF(OR(I152=0,V152="IGEN",W152="IGEN"),0,IF(AND(K152&lt;&gt;"IGEN",L152="IGEN",U152="NEM"),0,S152)))</f>
+        <f>IF(S152="","",IF(OR(I152=0,V152="IGEN",W152="IGEN"),0,IF(AND(K152&lt;&gt;"IGEN",L152="IGEN",U152="NEM"),0,IF(AND(H152="GYES",E152&lt;1998),0,S152))))</f>
         <v/>
       </c>
       <c r="AI152" s="6">
@@ -30159,7 +30159,7 @@
         <v/>
       </c>
       <c r="AH153" s="6">
-        <f>IF(S153="","",IF(OR(I153=0,V153="IGEN",W153="IGEN"),0,IF(AND(K153&lt;&gt;"IGEN",L153="IGEN",U153="NEM"),0,S153)))</f>
+        <f>IF(S153="","",IF(OR(I153=0,V153="IGEN",W153="IGEN"),0,IF(AND(K153&lt;&gt;"IGEN",L153="IGEN",U153="NEM"),0,IF(AND(H153="GYES",E153&lt;1998),0,S153))))</f>
         <v/>
       </c>
       <c r="AI153" s="6">
@@ -30279,7 +30279,7 @@
         <v/>
       </c>
       <c r="AH154" s="6">
-        <f>IF(S154="","",IF(OR(I154=0,V154="IGEN",W154="IGEN"),0,IF(AND(K154&lt;&gt;"IGEN",L154="IGEN",U154="NEM"),0,S154)))</f>
+        <f>IF(S154="","",IF(OR(I154=0,V154="IGEN",W154="IGEN"),0,IF(AND(K154&lt;&gt;"IGEN",L154="IGEN",U154="NEM"),0,IF(AND(H154="GYES",E154&lt;1998),0,S154))))</f>
         <v/>
       </c>
       <c r="AI154" s="6">
@@ -30399,7 +30399,7 @@
         <v/>
       </c>
       <c r="AH155" s="6">
-        <f>IF(S155="","",IF(OR(I155=0,V155="IGEN",W155="IGEN"),0,IF(AND(K155&lt;&gt;"IGEN",L155="IGEN",U155="NEM"),0,S155)))</f>
+        <f>IF(S155="","",IF(OR(I155=0,V155="IGEN",W155="IGEN"),0,IF(AND(K155&lt;&gt;"IGEN",L155="IGEN",U155="NEM"),0,IF(AND(H155="GYES",E155&lt;1998),0,S155))))</f>
         <v/>
       </c>
       <c r="AI155" s="6">
@@ -30519,7 +30519,7 @@
         <v/>
       </c>
       <c r="AH156" s="6">
-        <f>IF(S156="","",IF(OR(I156=0,V156="IGEN",W156="IGEN"),0,IF(AND(K156&lt;&gt;"IGEN",L156="IGEN",U156="NEM"),0,S156)))</f>
+        <f>IF(S156="","",IF(OR(I156=0,V156="IGEN",W156="IGEN"),0,IF(AND(K156&lt;&gt;"IGEN",L156="IGEN",U156="NEM"),0,IF(AND(H156="GYES",E156&lt;1998),0,S156))))</f>
         <v/>
       </c>
       <c r="AI156" s="6">
@@ -30639,7 +30639,7 @@
         <v/>
       </c>
       <c r="AH157" s="6">
-        <f>IF(S157="","",IF(OR(I157=0,V157="IGEN",W157="IGEN"),0,IF(AND(K157&lt;&gt;"IGEN",L157="IGEN",U157="NEM"),0,S157)))</f>
+        <f>IF(S157="","",IF(OR(I157=0,V157="IGEN",W157="IGEN"),0,IF(AND(K157&lt;&gt;"IGEN",L157="IGEN",U157="NEM"),0,IF(AND(H157="GYES",E157&lt;1998),0,S157))))</f>
         <v/>
       </c>
       <c r="AI157" s="6">
@@ -30759,7 +30759,7 @@
         <v/>
       </c>
       <c r="AH158" s="6">
-        <f>IF(S158="","",IF(OR(I158=0,V158="IGEN",W158="IGEN"),0,IF(AND(K158&lt;&gt;"IGEN",L158="IGEN",U158="NEM"),0,S158)))</f>
+        <f>IF(S158="","",IF(OR(I158=0,V158="IGEN",W158="IGEN"),0,IF(AND(K158&lt;&gt;"IGEN",L158="IGEN",U158="NEM"),0,IF(AND(H158="GYES",E158&lt;1998),0,S158))))</f>
         <v/>
       </c>
       <c r="AI158" s="6">
@@ -30879,7 +30879,7 @@
         <v/>
       </c>
       <c r="AH159" s="6">
-        <f>IF(S159="","",IF(OR(I159=0,V159="IGEN",W159="IGEN"),0,IF(AND(K159&lt;&gt;"IGEN",L159="IGEN",U159="NEM"),0,S159)))</f>
+        <f>IF(S159="","",IF(OR(I159=0,V159="IGEN",W159="IGEN"),0,IF(AND(K159&lt;&gt;"IGEN",L159="IGEN",U159="NEM"),0,IF(AND(H159="GYES",E159&lt;1998),0,S159))))</f>
         <v/>
       </c>
       <c r="AI159" s="6">
@@ -30999,7 +30999,7 @@
         <v/>
       </c>
       <c r="AH160" s="6">
-        <f>IF(S160="","",IF(OR(I160=0,V160="IGEN",W160="IGEN"),0,IF(AND(K160&lt;&gt;"IGEN",L160="IGEN",U160="NEM"),0,S160)))</f>
+        <f>IF(S160="","",IF(OR(I160=0,V160="IGEN",W160="IGEN"),0,IF(AND(K160&lt;&gt;"IGEN",L160="IGEN",U160="NEM"),0,IF(AND(H160="GYES",E160&lt;1998),0,S160))))</f>
         <v/>
       </c>
       <c r="AI160" s="6">
@@ -31119,7 +31119,7 @@
         <v/>
       </c>
       <c r="AH161" s="6">
-        <f>IF(S161="","",IF(OR(I161=0,V161="IGEN",W161="IGEN"),0,IF(AND(K161&lt;&gt;"IGEN",L161="IGEN",U161="NEM"),0,S161)))</f>
+        <f>IF(S161="","",IF(OR(I161=0,V161="IGEN",W161="IGEN"),0,IF(AND(K161&lt;&gt;"IGEN",L161="IGEN",U161="NEM"),0,IF(AND(H161="GYES",E161&lt;1998),0,S161))))</f>
         <v/>
       </c>
       <c r="AI161" s="6">
@@ -31239,7 +31239,7 @@
         <v/>
       </c>
       <c r="AH162" s="6">
-        <f>IF(S162="","",IF(OR(I162=0,V162="IGEN",W162="IGEN"),0,IF(AND(K162&lt;&gt;"IGEN",L162="IGEN",U162="NEM"),0,S162)))</f>
+        <f>IF(S162="","",IF(OR(I162=0,V162="IGEN",W162="IGEN"),0,IF(AND(K162&lt;&gt;"IGEN",L162="IGEN",U162="NEM"),0,IF(AND(H162="GYES",E162&lt;1998),0,S162))))</f>
         <v/>
       </c>
       <c r="AI162" s="6">
@@ -31359,7 +31359,7 @@
         <v/>
       </c>
       <c r="AH163" s="6">
-        <f>IF(S163="","",IF(OR(I163=0,V163="IGEN",W163="IGEN"),0,IF(AND(K163&lt;&gt;"IGEN",L163="IGEN",U163="NEM"),0,S163)))</f>
+        <f>IF(S163="","",IF(OR(I163=0,V163="IGEN",W163="IGEN"),0,IF(AND(K163&lt;&gt;"IGEN",L163="IGEN",U163="NEM"),0,IF(AND(H163="GYES",E163&lt;1998),0,S163))))</f>
         <v/>
       </c>
       <c r="AI163" s="6">
@@ -31479,7 +31479,7 @@
         <v/>
       </c>
       <c r="AH164" s="6">
-        <f>IF(S164="","",IF(OR(I164=0,V164="IGEN",W164="IGEN"),0,IF(AND(K164&lt;&gt;"IGEN",L164="IGEN",U164="NEM"),0,S164)))</f>
+        <f>IF(S164="","",IF(OR(I164=0,V164="IGEN",W164="IGEN"),0,IF(AND(K164&lt;&gt;"IGEN",L164="IGEN",U164="NEM"),0,IF(AND(H164="GYES",E164&lt;1998),0,S164))))</f>
         <v/>
       </c>
       <c r="AI164" s="6">
@@ -31599,7 +31599,7 @@
         <v/>
       </c>
       <c r="AH165" s="6">
-        <f>IF(S165="","",IF(OR(I165=0,V165="IGEN",W165="IGEN"),0,IF(AND(K165&lt;&gt;"IGEN",L165="IGEN",U165="NEM"),0,S165)))</f>
+        <f>IF(S165="","",IF(OR(I165=0,V165="IGEN",W165="IGEN"),0,IF(AND(K165&lt;&gt;"IGEN",L165="IGEN",U165="NEM"),0,IF(AND(H165="GYES",E165&lt;1998),0,S165))))</f>
         <v/>
       </c>
       <c r="AI165" s="6">
@@ -31719,7 +31719,7 @@
         <v/>
       </c>
       <c r="AH166" s="6">
-        <f>IF(S166="","",IF(OR(I166=0,V166="IGEN",W166="IGEN"),0,IF(AND(K166&lt;&gt;"IGEN",L166="IGEN",U166="NEM"),0,S166)))</f>
+        <f>IF(S166="","",IF(OR(I166=0,V166="IGEN",W166="IGEN"),0,IF(AND(K166&lt;&gt;"IGEN",L166="IGEN",U166="NEM"),0,IF(AND(H166="GYES",E166&lt;1998),0,S166))))</f>
         <v/>
       </c>
       <c r="AI166" s="6">
@@ -31839,7 +31839,7 @@
         <v/>
       </c>
       <c r="AH167" s="6">
-        <f>IF(S167="","",IF(OR(I167=0,V167="IGEN",W167="IGEN"),0,IF(AND(K167&lt;&gt;"IGEN",L167="IGEN",U167="NEM"),0,S167)))</f>
+        <f>IF(S167="","",IF(OR(I167=0,V167="IGEN",W167="IGEN"),0,IF(AND(K167&lt;&gt;"IGEN",L167="IGEN",U167="NEM"),0,IF(AND(H167="GYES",E167&lt;1998),0,S167))))</f>
         <v/>
       </c>
       <c r="AI167" s="6">
@@ -31959,7 +31959,7 @@
         <v/>
       </c>
       <c r="AH168" s="6">
-        <f>IF(S168="","",IF(OR(I168=0,V168="IGEN",W168="IGEN"),0,IF(AND(K168&lt;&gt;"IGEN",L168="IGEN",U168="NEM"),0,S168)))</f>
+        <f>IF(S168="","",IF(OR(I168=0,V168="IGEN",W168="IGEN"),0,IF(AND(K168&lt;&gt;"IGEN",L168="IGEN",U168="NEM"),0,IF(AND(H168="GYES",E168&lt;1998),0,S168))))</f>
         <v/>
       </c>
       <c r="AI168" s="6">
@@ -32079,7 +32079,7 @@
         <v/>
       </c>
       <c r="AH169" s="6">
-        <f>IF(S169="","",IF(OR(I169=0,V169="IGEN",W169="IGEN"),0,IF(AND(K169&lt;&gt;"IGEN",L169="IGEN",U169="NEM"),0,S169)))</f>
+        <f>IF(S169="","",IF(OR(I169=0,V169="IGEN",W169="IGEN"),0,IF(AND(K169&lt;&gt;"IGEN",L169="IGEN",U169="NEM"),0,IF(AND(H169="GYES",E169&lt;1998),0,S169))))</f>
         <v/>
       </c>
       <c r="AI169" s="6">
@@ -32199,7 +32199,7 @@
         <v/>
       </c>
       <c r="AH170" s="6">
-        <f>IF(S170="","",IF(OR(I170=0,V170="IGEN",W170="IGEN"),0,IF(AND(K170&lt;&gt;"IGEN",L170="IGEN",U170="NEM"),0,S170)))</f>
+        <f>IF(S170="","",IF(OR(I170=0,V170="IGEN",W170="IGEN"),0,IF(AND(K170&lt;&gt;"IGEN",L170="IGEN",U170="NEM"),0,IF(AND(H170="GYES",E170&lt;1998),0,S170))))</f>
         <v/>
       </c>
       <c r="AI170" s="6">
@@ -32319,7 +32319,7 @@
         <v/>
       </c>
       <c r="AH171" s="6">
-        <f>IF(S171="","",IF(OR(I171=0,V171="IGEN",W171="IGEN"),0,IF(AND(K171&lt;&gt;"IGEN",L171="IGEN",U171="NEM"),0,S171)))</f>
+        <f>IF(S171="","",IF(OR(I171=0,V171="IGEN",W171="IGEN"),0,IF(AND(K171&lt;&gt;"IGEN",L171="IGEN",U171="NEM"),0,IF(AND(H171="GYES",E171&lt;1998),0,S171))))</f>
         <v/>
       </c>
       <c r="AI171" s="6">
@@ -32439,7 +32439,7 @@
         <v/>
       </c>
       <c r="AH172" s="6">
-        <f>IF(S172="","",IF(OR(I172=0,V172="IGEN",W172="IGEN"),0,IF(AND(K172&lt;&gt;"IGEN",L172="IGEN",U172="NEM"),0,S172)))</f>
+        <f>IF(S172="","",IF(OR(I172=0,V172="IGEN",W172="IGEN"),0,IF(AND(K172&lt;&gt;"IGEN",L172="IGEN",U172="NEM"),0,IF(AND(H172="GYES",E172&lt;1998),0,S172))))</f>
         <v/>
       </c>
       <c r="AI172" s="6">
@@ -32559,7 +32559,7 @@
         <v/>
       </c>
       <c r="AH173" s="6">
-        <f>IF(S173="","",IF(OR(I173=0,V173="IGEN",W173="IGEN"),0,IF(AND(K173&lt;&gt;"IGEN",L173="IGEN",U173="NEM"),0,S173)))</f>
+        <f>IF(S173="","",IF(OR(I173=0,V173="IGEN",W173="IGEN"),0,IF(AND(K173&lt;&gt;"IGEN",L173="IGEN",U173="NEM"),0,IF(AND(H173="GYES",E173&lt;1998),0,S173))))</f>
         <v/>
       </c>
       <c r="AI173" s="6">
@@ -32679,7 +32679,7 @@
         <v/>
       </c>
       <c r="AH174" s="6">
-        <f>IF(S174="","",IF(OR(I174=0,V174="IGEN",W174="IGEN"),0,IF(AND(K174&lt;&gt;"IGEN",L174="IGEN",U174="NEM"),0,S174)))</f>
+        <f>IF(S174="","",IF(OR(I174=0,V174="IGEN",W174="IGEN"),0,IF(AND(K174&lt;&gt;"IGEN",L174="IGEN",U174="NEM"),0,IF(AND(H174="GYES",E174&lt;1998),0,S174))))</f>
         <v/>
       </c>
       <c r="AI174" s="6">
@@ -32799,7 +32799,7 @@
         <v/>
       </c>
       <c r="AH175" s="6">
-        <f>IF(S175="","",IF(OR(I175=0,V175="IGEN",W175="IGEN"),0,IF(AND(K175&lt;&gt;"IGEN",L175="IGEN",U175="NEM"),0,S175)))</f>
+        <f>IF(S175="","",IF(OR(I175=0,V175="IGEN",W175="IGEN"),0,IF(AND(K175&lt;&gt;"IGEN",L175="IGEN",U175="NEM"),0,IF(AND(H175="GYES",E175&lt;1998),0,S175))))</f>
         <v/>
       </c>
       <c r="AI175" s="6">
@@ -32919,7 +32919,7 @@
         <v/>
       </c>
       <c r="AH176" s="6">
-        <f>IF(S176="","",IF(OR(I176=0,V176="IGEN",W176="IGEN"),0,IF(AND(K176&lt;&gt;"IGEN",L176="IGEN",U176="NEM"),0,S176)))</f>
+        <f>IF(S176="","",IF(OR(I176=0,V176="IGEN",W176="IGEN"),0,IF(AND(K176&lt;&gt;"IGEN",L176="IGEN",U176="NEM"),0,IF(AND(H176="GYES",E176&lt;1998),0,S176))))</f>
         <v/>
       </c>
       <c r="AI176" s="6">
@@ -33039,7 +33039,7 @@
         <v/>
       </c>
       <c r="AH177" s="6">
-        <f>IF(S177="","",IF(OR(I177=0,V177="IGEN",W177="IGEN"),0,IF(AND(K177&lt;&gt;"IGEN",L177="IGEN",U177="NEM"),0,S177)))</f>
+        <f>IF(S177="","",IF(OR(I177=0,V177="IGEN",W177="IGEN"),0,IF(AND(K177&lt;&gt;"IGEN",L177="IGEN",U177="NEM"),0,IF(AND(H177="GYES",E177&lt;1998),0,S177))))</f>
         <v/>
       </c>
       <c r="AI177" s="6">
@@ -33159,7 +33159,7 @@
         <v/>
       </c>
       <c r="AH178" s="6">
-        <f>IF(S178="","",IF(OR(I178=0,V178="IGEN",W178="IGEN"),0,IF(AND(K178&lt;&gt;"IGEN",L178="IGEN",U178="NEM"),0,S178)))</f>
+        <f>IF(S178="","",IF(OR(I178=0,V178="IGEN",W178="IGEN"),0,IF(AND(K178&lt;&gt;"IGEN",L178="IGEN",U178="NEM"),0,IF(AND(H178="GYES",E178&lt;1998),0,S178))))</f>
         <v/>
       </c>
       <c r="AI178" s="6">
@@ -33279,7 +33279,7 @@
         <v/>
       </c>
       <c r="AH179" s="6">
-        <f>IF(S179="","",IF(OR(I179=0,V179="IGEN",W179="IGEN"),0,IF(AND(K179&lt;&gt;"IGEN",L179="IGEN",U179="NEM"),0,S179)))</f>
+        <f>IF(S179="","",IF(OR(I179=0,V179="IGEN",W179="IGEN"),0,IF(AND(K179&lt;&gt;"IGEN",L179="IGEN",U179="NEM"),0,IF(AND(H179="GYES",E179&lt;1998),0,S179))))</f>
         <v/>
       </c>
       <c r="AI179" s="6">
@@ -33399,7 +33399,7 @@
         <v/>
       </c>
       <c r="AH180" s="6">
-        <f>IF(S180="","",IF(OR(I180=0,V180="IGEN",W180="IGEN"),0,IF(AND(K180&lt;&gt;"IGEN",L180="IGEN",U180="NEM"),0,S180)))</f>
+        <f>IF(S180="","",IF(OR(I180=0,V180="IGEN",W180="IGEN"),0,IF(AND(K180&lt;&gt;"IGEN",L180="IGEN",U180="NEM"),0,IF(AND(H180="GYES",E180&lt;1998),0,S180))))</f>
         <v/>
       </c>
       <c r="AI180" s="6">
@@ -33519,7 +33519,7 @@
         <v/>
       </c>
       <c r="AH181" s="6">
-        <f>IF(S181="","",IF(OR(I181=0,V181="IGEN",W181="IGEN"),0,IF(AND(K181&lt;&gt;"IGEN",L181="IGEN",U181="NEM"),0,S181)))</f>
+        <f>IF(S181="","",IF(OR(I181=0,V181="IGEN",W181="IGEN"),0,IF(AND(K181&lt;&gt;"IGEN",L181="IGEN",U181="NEM"),0,IF(AND(H181="GYES",E181&lt;1998),0,S181))))</f>
         <v/>
       </c>
       <c r="AI181" s="6">
@@ -33639,7 +33639,7 @@
         <v/>
       </c>
       <c r="AH182" s="6">
-        <f>IF(S182="","",IF(OR(I182=0,V182="IGEN",W182="IGEN"),0,IF(AND(K182&lt;&gt;"IGEN",L182="IGEN",U182="NEM"),0,S182)))</f>
+        <f>IF(S182="","",IF(OR(I182=0,V182="IGEN",W182="IGEN"),0,IF(AND(K182&lt;&gt;"IGEN",L182="IGEN",U182="NEM"),0,IF(AND(H182="GYES",E182&lt;1998),0,S182))))</f>
         <v/>
       </c>
       <c r="AI182" s="6">
@@ -33759,7 +33759,7 @@
         <v/>
       </c>
       <c r="AH183" s="6">
-        <f>IF(S183="","",IF(OR(I183=0,V183="IGEN",W183="IGEN"),0,IF(AND(K183&lt;&gt;"IGEN",L183="IGEN",U183="NEM"),0,S183)))</f>
+        <f>IF(S183="","",IF(OR(I183=0,V183="IGEN",W183="IGEN"),0,IF(AND(K183&lt;&gt;"IGEN",L183="IGEN",U183="NEM"),0,IF(AND(H183="GYES",E183&lt;1998),0,S183))))</f>
         <v/>
       </c>
       <c r="AI183" s="6">
@@ -33879,7 +33879,7 @@
         <v/>
       </c>
       <c r="AH184" s="6">
-        <f>IF(S184="","",IF(OR(I184=0,V184="IGEN",W184="IGEN"),0,IF(AND(K184&lt;&gt;"IGEN",L184="IGEN",U184="NEM"),0,S184)))</f>
+        <f>IF(S184="","",IF(OR(I184=0,V184="IGEN",W184="IGEN"),0,IF(AND(K184&lt;&gt;"IGEN",L184="IGEN",U184="NEM"),0,IF(AND(H184="GYES",E184&lt;1998),0,S184))))</f>
         <v/>
       </c>
       <c r="AI184" s="6">
@@ -33999,7 +33999,7 @@
         <v/>
       </c>
       <c r="AH185" s="6">
-        <f>IF(S185="","",IF(OR(I185=0,V185="IGEN",W185="IGEN"),0,IF(AND(K185&lt;&gt;"IGEN",L185="IGEN",U185="NEM"),0,S185)))</f>
+        <f>IF(S185="","",IF(OR(I185=0,V185="IGEN",W185="IGEN"),0,IF(AND(K185&lt;&gt;"IGEN",L185="IGEN",U185="NEM"),0,IF(AND(H185="GYES",E185&lt;1998),0,S185))))</f>
         <v/>
       </c>
       <c r="AI185" s="6">
@@ -34119,7 +34119,7 @@
         <v/>
       </c>
       <c r="AH186" s="6">
-        <f>IF(S186="","",IF(OR(I186=0,V186="IGEN",W186="IGEN"),0,IF(AND(K186&lt;&gt;"IGEN",L186="IGEN",U186="NEM"),0,S186)))</f>
+        <f>IF(S186="","",IF(OR(I186=0,V186="IGEN",W186="IGEN"),0,IF(AND(K186&lt;&gt;"IGEN",L186="IGEN",U186="NEM"),0,IF(AND(H186="GYES",E186&lt;1998),0,S186))))</f>
         <v/>
       </c>
       <c r="AI186" s="6">
@@ -34239,7 +34239,7 @@
         <v/>
       </c>
       <c r="AH187" s="6">
-        <f>IF(S187="","",IF(OR(I187=0,V187="IGEN",W187="IGEN"),0,IF(AND(K187&lt;&gt;"IGEN",L187="IGEN",U187="NEM"),0,S187)))</f>
+        <f>IF(S187="","",IF(OR(I187=0,V187="IGEN",W187="IGEN"),0,IF(AND(K187&lt;&gt;"IGEN",L187="IGEN",U187="NEM"),0,IF(AND(H187="GYES",E187&lt;1998),0,S187))))</f>
         <v/>
       </c>
       <c r="AI187" s="6">
@@ -34359,7 +34359,7 @@
         <v/>
       </c>
       <c r="AH188" s="6">
-        <f>IF(S188="","",IF(OR(I188=0,V188="IGEN",W188="IGEN"),0,IF(AND(K188&lt;&gt;"IGEN",L188="IGEN",U188="NEM"),0,S188)))</f>
+        <f>IF(S188="","",IF(OR(I188=0,V188="IGEN",W188="IGEN"),0,IF(AND(K188&lt;&gt;"IGEN",L188="IGEN",U188="NEM"),0,IF(AND(H188="GYES",E188&lt;1998),0,S188))))</f>
         <v/>
       </c>
       <c r="AI188" s="6">
@@ -34479,7 +34479,7 @@
         <v/>
       </c>
       <c r="AH189" s="6">
-        <f>IF(S189="","",IF(OR(I189=0,V189="IGEN",W189="IGEN"),0,IF(AND(K189&lt;&gt;"IGEN",L189="IGEN",U189="NEM"),0,S189)))</f>
+        <f>IF(S189="","",IF(OR(I189=0,V189="IGEN",W189="IGEN"),0,IF(AND(K189&lt;&gt;"IGEN",L189="IGEN",U189="NEM"),0,IF(AND(H189="GYES",E189&lt;1998),0,S189))))</f>
         <v/>
       </c>
       <c r="AI189" s="6">
@@ -34599,7 +34599,7 @@
         <v/>
       </c>
       <c r="AH190" s="6">
-        <f>IF(S190="","",IF(OR(I190=0,V190="IGEN",W190="IGEN"),0,IF(AND(K190&lt;&gt;"IGEN",L190="IGEN",U190="NEM"),0,S190)))</f>
+        <f>IF(S190="","",IF(OR(I190=0,V190="IGEN",W190="IGEN"),0,IF(AND(K190&lt;&gt;"IGEN",L190="IGEN",U190="NEM"),0,IF(AND(H190="GYES",E190&lt;1998),0,S190))))</f>
         <v/>
       </c>
       <c r="AI190" s="6">
@@ -34719,7 +34719,7 @@
         <v/>
       </c>
       <c r="AH191" s="6">
-        <f>IF(S191="","",IF(OR(I191=0,V191="IGEN",W191="IGEN"),0,IF(AND(K191&lt;&gt;"IGEN",L191="IGEN",U191="NEM"),0,S191)))</f>
+        <f>IF(S191="","",IF(OR(I191=0,V191="IGEN",W191="IGEN"),0,IF(AND(K191&lt;&gt;"IGEN",L191="IGEN",U191="NEM"),0,IF(AND(H191="GYES",E191&lt;1998),0,S191))))</f>
         <v/>
       </c>
       <c r="AI191" s="6">
@@ -34839,7 +34839,7 @@
         <v/>
       </c>
       <c r="AH192" s="6">
-        <f>IF(S192="","",IF(OR(I192=0,V192="IGEN",W192="IGEN"),0,IF(AND(K192&lt;&gt;"IGEN",L192="IGEN",U192="NEM"),0,S192)))</f>
+        <f>IF(S192="","",IF(OR(I192=0,V192="IGEN",W192="IGEN"),0,IF(AND(K192&lt;&gt;"IGEN",L192="IGEN",U192="NEM"),0,IF(AND(H192="GYES",E192&lt;1998),0,S192))))</f>
         <v/>
       </c>
       <c r="AI192" s="6">
@@ -34959,7 +34959,7 @@
         <v/>
       </c>
       <c r="AH193" s="6">
-        <f>IF(S193="","",IF(OR(I193=0,V193="IGEN",W193="IGEN"),0,IF(AND(K193&lt;&gt;"IGEN",L193="IGEN",U193="NEM"),0,S193)))</f>
+        <f>IF(S193="","",IF(OR(I193=0,V193="IGEN",W193="IGEN"),0,IF(AND(K193&lt;&gt;"IGEN",L193="IGEN",U193="NEM"),0,IF(AND(H193="GYES",E193&lt;1998),0,S193))))</f>
         <v/>
       </c>
       <c r="AI193" s="6">
@@ -35079,7 +35079,7 @@
         <v/>
       </c>
       <c r="AH194" s="6">
-        <f>IF(S194="","",IF(OR(I194=0,V194="IGEN",W194="IGEN"),0,IF(AND(K194&lt;&gt;"IGEN",L194="IGEN",U194="NEM"),0,S194)))</f>
+        <f>IF(S194="","",IF(OR(I194=0,V194="IGEN",W194="IGEN"),0,IF(AND(K194&lt;&gt;"IGEN",L194="IGEN",U194="NEM"),0,IF(AND(H194="GYES",E194&lt;1998),0,S194))))</f>
         <v/>
       </c>
       <c r="AI194" s="6">
@@ -35199,7 +35199,7 @@
         <v/>
       </c>
       <c r="AH195" s="6">
-        <f>IF(S195="","",IF(OR(I195=0,V195="IGEN",W195="IGEN"),0,IF(AND(K195&lt;&gt;"IGEN",L195="IGEN",U195="NEM"),0,S195)))</f>
+        <f>IF(S195="","",IF(OR(I195=0,V195="IGEN",W195="IGEN"),0,IF(AND(K195&lt;&gt;"IGEN",L195="IGEN",U195="NEM"),0,IF(AND(H195="GYES",E195&lt;1998),0,S195))))</f>
         <v/>
       </c>
       <c r="AI195" s="6">
@@ -35319,7 +35319,7 @@
         <v/>
       </c>
       <c r="AH196" s="6">
-        <f>IF(S196="","",IF(OR(I196=0,V196="IGEN",W196="IGEN"),0,IF(AND(K196&lt;&gt;"IGEN",L196="IGEN",U196="NEM"),0,S196)))</f>
+        <f>IF(S196="","",IF(OR(I196=0,V196="IGEN",W196="IGEN"),0,IF(AND(K196&lt;&gt;"IGEN",L196="IGEN",U196="NEM"),0,IF(AND(H196="GYES",E196&lt;1998),0,S196))))</f>
         <v/>
       </c>
       <c r="AI196" s="6">
@@ -35439,7 +35439,7 @@
         <v/>
       </c>
       <c r="AH197" s="6">
-        <f>IF(S197="","",IF(OR(I197=0,V197="IGEN",W197="IGEN"),0,IF(AND(K197&lt;&gt;"IGEN",L197="IGEN",U197="NEM"),0,S197)))</f>
+        <f>IF(S197="","",IF(OR(I197=0,V197="IGEN",W197="IGEN"),0,IF(AND(K197&lt;&gt;"IGEN",L197="IGEN",U197="NEM"),0,IF(AND(H197="GYES",E197&lt;1998),0,S197))))</f>
         <v/>
       </c>
       <c r="AI197" s="6">
@@ -35559,7 +35559,7 @@
         <v/>
       </c>
       <c r="AH198" s="6">
-        <f>IF(S198="","",IF(OR(I198=0,V198="IGEN",W198="IGEN"),0,IF(AND(K198&lt;&gt;"IGEN",L198="IGEN",U198="NEM"),0,S198)))</f>
+        <f>IF(S198="","",IF(OR(I198=0,V198="IGEN",W198="IGEN"),0,IF(AND(K198&lt;&gt;"IGEN",L198="IGEN",U198="NEM"),0,IF(AND(H198="GYES",E198&lt;1998),0,S198))))</f>
         <v/>
       </c>
       <c r="AI198" s="6">
@@ -35679,7 +35679,7 @@
         <v/>
       </c>
       <c r="AH199" s="6">
-        <f>IF(S199="","",IF(OR(I199=0,V199="IGEN",W199="IGEN"),0,IF(AND(K199&lt;&gt;"IGEN",L199="IGEN",U199="NEM"),0,S199)))</f>
+        <f>IF(S199="","",IF(OR(I199=0,V199="IGEN",W199="IGEN"),0,IF(AND(K199&lt;&gt;"IGEN",L199="IGEN",U199="NEM"),0,IF(AND(H199="GYES",E199&lt;1998),0,S199))))</f>
         <v/>
       </c>
       <c r="AI199" s="6">
@@ -35799,7 +35799,7 @@
         <v/>
       </c>
       <c r="AH200" s="6">
-        <f>IF(S200="","",IF(OR(I200=0,V200="IGEN",W200="IGEN"),0,IF(AND(K200&lt;&gt;"IGEN",L200="IGEN",U200="NEM"),0,S200)))</f>
+        <f>IF(S200="","",IF(OR(I200=0,V200="IGEN",W200="IGEN"),0,IF(AND(K200&lt;&gt;"IGEN",L200="IGEN",U200="NEM"),0,IF(AND(H200="GYES",E200&lt;1998),0,S200))))</f>
         <v/>
       </c>
       <c r="AI200" s="6">
@@ -35919,7 +35919,7 @@
         <v/>
       </c>
       <c r="AH201" s="6">
-        <f>IF(S201="","",IF(OR(I201=0,V201="IGEN",W201="IGEN"),0,IF(AND(K201&lt;&gt;"IGEN",L201="IGEN",U201="NEM"),0,S201)))</f>
+        <f>IF(S201="","",IF(OR(I201=0,V201="IGEN",W201="IGEN"),0,IF(AND(K201&lt;&gt;"IGEN",L201="IGEN",U201="NEM"),0,IF(AND(H201="GYES",E201&lt;1998),0,S201))))</f>
         <v/>
       </c>
       <c r="AI201" s="6">
@@ -36039,7 +36039,7 @@
         <v/>
       </c>
       <c r="AH202" s="6">
-        <f>IF(S202="","",IF(OR(I202=0,V202="IGEN",W202="IGEN"),0,IF(AND(K202&lt;&gt;"IGEN",L202="IGEN",U202="NEM"),0,S202)))</f>
+        <f>IF(S202="","",IF(OR(I202=0,V202="IGEN",W202="IGEN"),0,IF(AND(K202&lt;&gt;"IGEN",L202="IGEN",U202="NEM"),0,IF(AND(H202="GYES",E202&lt;1998),0,S202))))</f>
         <v/>
       </c>
       <c r="AI202" s="6">
@@ -36159,7 +36159,7 @@
         <v/>
       </c>
       <c r="AH203" s="6">
-        <f>IF(S203="","",IF(OR(I203=0,V203="IGEN",W203="IGEN"),0,IF(AND(K203&lt;&gt;"IGEN",L203="IGEN",U203="NEM"),0,S203)))</f>
+        <f>IF(S203="","",IF(OR(I203=0,V203="IGEN",W203="IGEN"),0,IF(AND(K203&lt;&gt;"IGEN",L203="IGEN",U203="NEM"),0,IF(AND(H203="GYES",E203&lt;1998),0,S203))))</f>
         <v/>
       </c>
       <c r="AI203" s="6">
@@ -36279,7 +36279,7 @@
         <v/>
       </c>
       <c r="AH204" s="6">
-        <f>IF(S204="","",IF(OR(I204=0,V204="IGEN",W204="IGEN"),0,IF(AND(K204&lt;&gt;"IGEN",L204="IGEN",U204="NEM"),0,S204)))</f>
+        <f>IF(S204="","",IF(OR(I204=0,V204="IGEN",W204="IGEN"),0,IF(AND(K204&lt;&gt;"IGEN",L204="IGEN",U204="NEM"),0,IF(AND(H204="GYES",E204&lt;1998),0,S204))))</f>
         <v/>
       </c>
       <c r="AI204" s="6">
@@ -36399,7 +36399,7 @@
         <v/>
       </c>
       <c r="AH205" s="6">
-        <f>IF(S205="","",IF(OR(I205=0,V205="IGEN",W205="IGEN"),0,IF(AND(K205&lt;&gt;"IGEN",L205="IGEN",U205="NEM"),0,S205)))</f>
+        <f>IF(S205="","",IF(OR(I205=0,V205="IGEN",W205="IGEN"),0,IF(AND(K205&lt;&gt;"IGEN",L205="IGEN",U205="NEM"),0,IF(AND(H205="GYES",E205&lt;1998),0,S205))))</f>
         <v/>
       </c>
       <c r="AI205" s="6">
@@ -36519,7 +36519,7 @@
         <v/>
       </c>
       <c r="AH206" s="6">
-        <f>IF(S206="","",IF(OR(I206=0,V206="IGEN",W206="IGEN"),0,IF(AND(K206&lt;&gt;"IGEN",L206="IGEN",U206="NEM"),0,S206)))</f>
+        <f>IF(S206="","",IF(OR(I206=0,V206="IGEN",W206="IGEN"),0,IF(AND(K206&lt;&gt;"IGEN",L206="IGEN",U206="NEM"),0,IF(AND(H206="GYES",E206&lt;1998),0,S206))))</f>
         <v/>
       </c>
       <c r="AI206" s="6">
@@ -36639,7 +36639,7 @@
         <v/>
       </c>
       <c r="AH207" s="6">
-        <f>IF(S207="","",IF(OR(I207=0,V207="IGEN",W207="IGEN"),0,IF(AND(K207&lt;&gt;"IGEN",L207="IGEN",U207="NEM"),0,S207)))</f>
+        <f>IF(S207="","",IF(OR(I207=0,V207="IGEN",W207="IGEN"),0,IF(AND(K207&lt;&gt;"IGEN",L207="IGEN",U207="NEM"),0,IF(AND(H207="GYES",E207&lt;1998),0,S207))))</f>
         <v/>
       </c>
       <c r="AI207" s="6">
@@ -36759,7 +36759,7 @@
         <v/>
       </c>
       <c r="AH208" s="6">
-        <f>IF(S208="","",IF(OR(I208=0,V208="IGEN",W208="IGEN"),0,IF(AND(K208&lt;&gt;"IGEN",L208="IGEN",U208="NEM"),0,S208)))</f>
+        <f>IF(S208="","",IF(OR(I208=0,V208="IGEN",W208="IGEN"),0,IF(AND(K208&lt;&gt;"IGEN",L208="IGEN",U208="NEM"),0,IF(AND(H208="GYES",E208&lt;1998),0,S208))))</f>
         <v/>
       </c>
       <c r="AI208" s="6">
@@ -36879,7 +36879,7 @@
         <v/>
       </c>
       <c r="AH209" s="6">
-        <f>IF(S209="","",IF(OR(I209=0,V209="IGEN",W209="IGEN"),0,IF(AND(K209&lt;&gt;"IGEN",L209="IGEN",U209="NEM"),0,S209)))</f>
+        <f>IF(S209="","",IF(OR(I209=0,V209="IGEN",W209="IGEN"),0,IF(AND(K209&lt;&gt;"IGEN",L209="IGEN",U209="NEM"),0,IF(AND(H209="GYES",E209&lt;1998),0,S209))))</f>
         <v/>
       </c>
       <c r="AI209" s="6">
@@ -36999,7 +36999,7 @@
         <v/>
       </c>
       <c r="AH210" s="6">
-        <f>IF(S210="","",IF(OR(I210=0,V210="IGEN",W210="IGEN"),0,IF(AND(K210&lt;&gt;"IGEN",L210="IGEN",U210="NEM"),0,S210)))</f>
+        <f>IF(S210="","",IF(OR(I210=0,V210="IGEN",W210="IGEN"),0,IF(AND(K210&lt;&gt;"IGEN",L210="IGEN",U210="NEM"),0,IF(AND(H210="GYES",E210&lt;1998),0,S210))))</f>
         <v/>
       </c>
       <c r="AI210" s="6">
@@ -37119,7 +37119,7 @@
         <v/>
       </c>
       <c r="AH211" s="6">
-        <f>IF(S211="","",IF(OR(I211=0,V211="IGEN",W211="IGEN"),0,IF(AND(K211&lt;&gt;"IGEN",L211="IGEN",U211="NEM"),0,S211)))</f>
+        <f>IF(S211="","",IF(OR(I211=0,V211="IGEN",W211="IGEN"),0,IF(AND(K211&lt;&gt;"IGEN",L211="IGEN",U211="NEM"),0,IF(AND(H211="GYES",E211&lt;1998),0,S211))))</f>
         <v/>
       </c>
       <c r="AI211" s="6">
@@ -37239,7 +37239,7 @@
         <v/>
       </c>
       <c r="AH212" s="6">
-        <f>IF(S212="","",IF(OR(I212=0,V212="IGEN",W212="IGEN"),0,IF(AND(K212&lt;&gt;"IGEN",L212="IGEN",U212="NEM"),0,S212)))</f>
+        <f>IF(S212="","",IF(OR(I212=0,V212="IGEN",W212="IGEN"),0,IF(AND(K212&lt;&gt;"IGEN",L212="IGEN",U212="NEM"),0,IF(AND(H212="GYES",E212&lt;1998),0,S212))))</f>
         <v/>
       </c>
       <c r="AI212" s="6">
@@ -37359,7 +37359,7 @@
         <v/>
       </c>
       <c r="AH213" s="6">
-        <f>IF(S213="","",IF(OR(I213=0,V213="IGEN",W213="IGEN"),0,IF(AND(K213&lt;&gt;"IGEN",L213="IGEN",U213="NEM"),0,S213)))</f>
+        <f>IF(S213="","",IF(OR(I213=0,V213="IGEN",W213="IGEN"),0,IF(AND(K213&lt;&gt;"IGEN",L213="IGEN",U213="NEM"),0,IF(AND(H213="GYES",E213&lt;1998),0,S213))))</f>
         <v/>
       </c>
       <c r="AI213" s="6">
@@ -37479,7 +37479,7 @@
         <v/>
       </c>
       <c r="AH214" s="6">
-        <f>IF(S214="","",IF(OR(I214=0,V214="IGEN",W214="IGEN"),0,IF(AND(K214&lt;&gt;"IGEN",L214="IGEN",U214="NEM"),0,S214)))</f>
+        <f>IF(S214="","",IF(OR(I214=0,V214="IGEN",W214="IGEN"),0,IF(AND(K214&lt;&gt;"IGEN",L214="IGEN",U214="NEM"),0,IF(AND(H214="GYES",E214&lt;1998),0,S214))))</f>
         <v/>
       </c>
       <c r="AI214" s="6">
@@ -37599,7 +37599,7 @@
         <v/>
       </c>
       <c r="AH215" s="6">
-        <f>IF(S215="","",IF(OR(I215=0,V215="IGEN",W215="IGEN"),0,IF(AND(K215&lt;&gt;"IGEN",L215="IGEN",U215="NEM"),0,S215)))</f>
+        <f>IF(S215="","",IF(OR(I215=0,V215="IGEN",W215="IGEN"),0,IF(AND(K215&lt;&gt;"IGEN",L215="IGEN",U215="NEM"),0,IF(AND(H215="GYES",E215&lt;1998),0,S215))))</f>
         <v/>
       </c>
       <c r="AI215" s="6">
@@ -37719,7 +37719,7 @@
         <v/>
       </c>
       <c r="AH216" s="6">
-        <f>IF(S216="","",IF(OR(I216=0,V216="IGEN",W216="IGEN"),0,IF(AND(K216&lt;&gt;"IGEN",L216="IGEN",U216="NEM"),0,S216)))</f>
+        <f>IF(S216="","",IF(OR(I216=0,V216="IGEN",W216="IGEN"),0,IF(AND(K216&lt;&gt;"IGEN",L216="IGEN",U216="NEM"),0,IF(AND(H216="GYES",E216&lt;1998),0,S216))))</f>
         <v/>
       </c>
       <c r="AI216" s="6">
@@ -37839,7 +37839,7 @@
         <v/>
       </c>
       <c r="AH217" s="6">
-        <f>IF(S217="","",IF(OR(I217=0,V217="IGEN",W217="IGEN"),0,IF(AND(K217&lt;&gt;"IGEN",L217="IGEN",U217="NEM"),0,S217)))</f>
+        <f>IF(S217="","",IF(OR(I217=0,V217="IGEN",W217="IGEN"),0,IF(AND(K217&lt;&gt;"IGEN",L217="IGEN",U217="NEM"),0,IF(AND(H217="GYES",E217&lt;1998),0,S217))))</f>
         <v/>
       </c>
       <c r="AI217" s="6">
@@ -37959,7 +37959,7 @@
         <v/>
       </c>
       <c r="AH218" s="6">
-        <f>IF(S218="","",IF(OR(I218=0,V218="IGEN",W218="IGEN"),0,IF(AND(K218&lt;&gt;"IGEN",L218="IGEN",U218="NEM"),0,S218)))</f>
+        <f>IF(S218="","",IF(OR(I218=0,V218="IGEN",W218="IGEN"),0,IF(AND(K218&lt;&gt;"IGEN",L218="IGEN",U218="NEM"),0,IF(AND(H218="GYES",E218&lt;1998),0,S218))))</f>
         <v/>
       </c>
       <c r="AI218" s="6">
@@ -38079,7 +38079,7 @@
         <v/>
       </c>
       <c r="AH219" s="6">
-        <f>IF(S219="","",IF(OR(I219=0,V219="IGEN",W219="IGEN"),0,IF(AND(K219&lt;&gt;"IGEN",L219="IGEN",U219="NEM"),0,S219)))</f>
+        <f>IF(S219="","",IF(OR(I219=0,V219="IGEN",W219="IGEN"),0,IF(AND(K219&lt;&gt;"IGEN",L219="IGEN",U219="NEM"),0,IF(AND(H219="GYES",E219&lt;1998),0,S219))))</f>
         <v/>
       </c>
       <c r="AI219" s="6">
@@ -38199,7 +38199,7 @@
         <v/>
       </c>
       <c r="AH220" s="6">
-        <f>IF(S220="","",IF(OR(I220=0,V220="IGEN",W220="IGEN"),0,IF(AND(K220&lt;&gt;"IGEN",L220="IGEN",U220="NEM"),0,S220)))</f>
+        <f>IF(S220="","",IF(OR(I220=0,V220="IGEN",W220="IGEN"),0,IF(AND(K220&lt;&gt;"IGEN",L220="IGEN",U220="NEM"),0,IF(AND(H220="GYES",E220&lt;1998),0,S220))))</f>
         <v/>
       </c>
       <c r="AI220" s="6">
@@ -38319,7 +38319,7 @@
         <v/>
       </c>
       <c r="AH221" s="6">
-        <f>IF(S221="","",IF(OR(I221=0,V221="IGEN",W221="IGEN"),0,IF(AND(K221&lt;&gt;"IGEN",L221="IGEN",U221="NEM"),0,S221)))</f>
+        <f>IF(S221="","",IF(OR(I221=0,V221="IGEN",W221="IGEN"),0,IF(AND(K221&lt;&gt;"IGEN",L221="IGEN",U221="NEM"),0,IF(AND(H221="GYES",E221&lt;1998),0,S221))))</f>
         <v/>
       </c>
       <c r="AI221" s="6">
@@ -38439,7 +38439,7 @@
         <v/>
       </c>
       <c r="AH222" s="6">
-        <f>IF(S222="","",IF(OR(I222=0,V222="IGEN",W222="IGEN"),0,IF(AND(K222&lt;&gt;"IGEN",L222="IGEN",U222="NEM"),0,S222)))</f>
+        <f>IF(S222="","",IF(OR(I222=0,V222="IGEN",W222="IGEN"),0,IF(AND(K222&lt;&gt;"IGEN",L222="IGEN",U222="NEM"),0,IF(AND(H222="GYES",E222&lt;1998),0,S222))))</f>
         <v/>
       </c>
       <c r="AI222" s="6">
@@ -38559,7 +38559,7 @@
         <v/>
       </c>
       <c r="AH223" s="6">
-        <f>IF(S223="","",IF(OR(I223=0,V223="IGEN",W223="IGEN"),0,IF(AND(K223&lt;&gt;"IGEN",L223="IGEN",U223="NEM"),0,S223)))</f>
+        <f>IF(S223="","",IF(OR(I223=0,V223="IGEN",W223="IGEN"),0,IF(AND(K223&lt;&gt;"IGEN",L223="IGEN",U223="NEM"),0,IF(AND(H223="GYES",E223&lt;1998),0,S223))))</f>
         <v/>
       </c>
       <c r="AI223" s="6">
@@ -38679,7 +38679,7 @@
         <v/>
       </c>
       <c r="AH224" s="6">
-        <f>IF(S224="","",IF(OR(I224=0,V224="IGEN",W224="IGEN"),0,IF(AND(K224&lt;&gt;"IGEN",L224="IGEN",U224="NEM"),0,S224)))</f>
+        <f>IF(S224="","",IF(OR(I224=0,V224="IGEN",W224="IGEN"),0,IF(AND(K224&lt;&gt;"IGEN",L224="IGEN",U224="NEM"),0,IF(AND(H224="GYES",E224&lt;1998),0,S224))))</f>
         <v/>
       </c>
       <c r="AI224" s="6">
@@ -38799,7 +38799,7 @@
         <v/>
       </c>
       <c r="AH225" s="6">
-        <f>IF(S225="","",IF(OR(I225=0,V225="IGEN",W225="IGEN"),0,IF(AND(K225&lt;&gt;"IGEN",L225="IGEN",U225="NEM"),0,S225)))</f>
+        <f>IF(S225="","",IF(OR(I225=0,V225="IGEN",W225="IGEN"),0,IF(AND(K225&lt;&gt;"IGEN",L225="IGEN",U225="NEM"),0,IF(AND(H225="GYES",E225&lt;1998),0,S225))))</f>
         <v/>
       </c>
       <c r="AI225" s="6">
@@ -38919,7 +38919,7 @@
         <v/>
       </c>
       <c r="AH226" s="6">
-        <f>IF(S226="","",IF(OR(I226=0,V226="IGEN",W226="IGEN"),0,IF(AND(K226&lt;&gt;"IGEN",L226="IGEN",U226="NEM"),0,S226)))</f>
+        <f>IF(S226="","",IF(OR(I226=0,V226="IGEN",W226="IGEN"),0,IF(AND(K226&lt;&gt;"IGEN",L226="IGEN",U226="NEM"),0,IF(AND(H226="GYES",E226&lt;1998),0,S226))))</f>
         <v/>
       </c>
       <c r="AI226" s="6">
@@ -39039,7 +39039,7 @@
         <v/>
       </c>
       <c r="AH227" s="6">
-        <f>IF(S227="","",IF(OR(I227=0,V227="IGEN",W227="IGEN"),0,IF(AND(K227&lt;&gt;"IGEN",L227="IGEN",U227="NEM"),0,S227)))</f>
+        <f>IF(S227="","",IF(OR(I227=0,V227="IGEN",W227="IGEN"),0,IF(AND(K227&lt;&gt;"IGEN",L227="IGEN",U227="NEM"),0,IF(AND(H227="GYES",E227&lt;1998),0,S227))))</f>
         <v/>
       </c>
       <c r="AI227" s="6">
@@ -39159,7 +39159,7 @@
         <v/>
       </c>
       <c r="AH228" s="6">
-        <f>IF(S228="","",IF(OR(I228=0,V228="IGEN",W228="IGEN"),0,IF(AND(K228&lt;&gt;"IGEN",L228="IGEN",U228="NEM"),0,S228)))</f>
+        <f>IF(S228="","",IF(OR(I228=0,V228="IGEN",W228="IGEN"),0,IF(AND(K228&lt;&gt;"IGEN",L228="IGEN",U228="NEM"),0,IF(AND(H228="GYES",E228&lt;1998),0,S228))))</f>
         <v/>
       </c>
       <c r="AI228" s="6">
@@ -39279,7 +39279,7 @@
         <v/>
       </c>
       <c r="AH229" s="6">
-        <f>IF(S229="","",IF(OR(I229=0,V229="IGEN",W229="IGEN"),0,IF(AND(K229&lt;&gt;"IGEN",L229="IGEN",U229="NEM"),0,S229)))</f>
+        <f>IF(S229="","",IF(OR(I229=0,V229="IGEN",W229="IGEN"),0,IF(AND(K229&lt;&gt;"IGEN",L229="IGEN",U229="NEM"),0,IF(AND(H229="GYES",E229&lt;1998),0,S229))))</f>
         <v/>
       </c>
       <c r="AI229" s="6">
@@ -39399,7 +39399,7 @@
         <v/>
       </c>
       <c r="AH230" s="6">
-        <f>IF(S230="","",IF(OR(I230=0,V230="IGEN",W230="IGEN"),0,IF(AND(K230&lt;&gt;"IGEN",L230="IGEN",U230="NEM"),0,S230)))</f>
+        <f>IF(S230="","",IF(OR(I230=0,V230="IGEN",W230="IGEN"),0,IF(AND(K230&lt;&gt;"IGEN",L230="IGEN",U230="NEM"),0,IF(AND(H230="GYES",E230&lt;1998),0,S230))))</f>
         <v/>
       </c>
       <c r="AI230" s="6">
@@ -39519,7 +39519,7 @@
         <v/>
       </c>
       <c r="AH231" s="6">
-        <f>IF(S231="","",IF(OR(I231=0,V231="IGEN",W231="IGEN"),0,IF(AND(K231&lt;&gt;"IGEN",L231="IGEN",U231="NEM"),0,S231)))</f>
+        <f>IF(S231="","",IF(OR(I231=0,V231="IGEN",W231="IGEN"),0,IF(AND(K231&lt;&gt;"IGEN",L231="IGEN",U231="NEM"),0,IF(AND(H231="GYES",E231&lt;1998),0,S231))))</f>
         <v/>
       </c>
       <c r="AI231" s="6">
@@ -39639,7 +39639,7 @@
         <v/>
       </c>
       <c r="AH232" s="6">
-        <f>IF(S232="","",IF(OR(I232=0,V232="IGEN",W232="IGEN"),0,IF(AND(K232&lt;&gt;"IGEN",L232="IGEN",U232="NEM"),0,S232)))</f>
+        <f>IF(S232="","",IF(OR(I232=0,V232="IGEN",W232="IGEN"),0,IF(AND(K232&lt;&gt;"IGEN",L232="IGEN",U232="NEM"),0,IF(AND(H232="GYES",E232&lt;1998),0,S232))))</f>
         <v/>
       </c>
       <c r="AI232" s="6">
@@ -39759,7 +39759,7 @@
         <v/>
       </c>
       <c r="AH233" s="6">
-        <f>IF(S233="","",IF(OR(I233=0,V233="IGEN",W233="IGEN"),0,IF(AND(K233&lt;&gt;"IGEN",L233="IGEN",U233="NEM"),0,S233)))</f>
+        <f>IF(S233="","",IF(OR(I233=0,V233="IGEN",W233="IGEN"),0,IF(AND(K233&lt;&gt;"IGEN",L233="IGEN",U233="NEM"),0,IF(AND(H233="GYES",E233&lt;1998),0,S233))))</f>
         <v/>
       </c>
       <c r="AI233" s="6">
@@ -39879,7 +39879,7 @@
         <v/>
       </c>
       <c r="AH234" s="6">
-        <f>IF(S234="","",IF(OR(I234=0,V234="IGEN",W234="IGEN"),0,IF(AND(K234&lt;&gt;"IGEN",L234="IGEN",U234="NEM"),0,S234)))</f>
+        <f>IF(S234="","",IF(OR(I234=0,V234="IGEN",W234="IGEN"),0,IF(AND(K234&lt;&gt;"IGEN",L234="IGEN",U234="NEM"),0,IF(AND(H234="GYES",E234&lt;1998),0,S234))))</f>
         <v/>
       </c>
       <c r="AI234" s="6">
@@ -39999,7 +39999,7 @@
         <v/>
       </c>
       <c r="AH235" s="6">
-        <f>IF(S235="","",IF(OR(I235=0,V235="IGEN",W235="IGEN"),0,IF(AND(K235&lt;&gt;"IGEN",L235="IGEN",U235="NEM"),0,S235)))</f>
+        <f>IF(S235="","",IF(OR(I235=0,V235="IGEN",W235="IGEN"),0,IF(AND(K235&lt;&gt;"IGEN",L235="IGEN",U235="NEM"),0,IF(AND(H235="GYES",E235&lt;1998),0,S235))))</f>
         <v/>
       </c>
       <c r="AI235" s="6">
@@ -40119,7 +40119,7 @@
         <v/>
       </c>
       <c r="AH236" s="6">
-        <f>IF(S236="","",IF(OR(I236=0,V236="IGEN",W236="IGEN"),0,IF(AND(K236&lt;&gt;"IGEN",L236="IGEN",U236="NEM"),0,S236)))</f>
+        <f>IF(S236="","",IF(OR(I236=0,V236="IGEN",W236="IGEN"),0,IF(AND(K236&lt;&gt;"IGEN",L236="IGEN",U236="NEM"),0,IF(AND(H236="GYES",E236&lt;1998),0,S236))))</f>
         <v/>
       </c>
       <c r="AI236" s="6">
@@ -40239,7 +40239,7 @@
         <v/>
       </c>
       <c r="AH237" s="6">
-        <f>IF(S237="","",IF(OR(I237=0,V237="IGEN",W237="IGEN"),0,IF(AND(K237&lt;&gt;"IGEN",L237="IGEN",U237="NEM"),0,S237)))</f>
+        <f>IF(S237="","",IF(OR(I237=0,V237="IGEN",W237="IGEN"),0,IF(AND(K237&lt;&gt;"IGEN",L237="IGEN",U237="NEM"),0,IF(AND(H237="GYES",E237&lt;1998),0,S237))))</f>
         <v/>
       </c>
       <c r="AI237" s="6">
@@ -40359,7 +40359,7 @@
         <v/>
       </c>
       <c r="AH238" s="6">
-        <f>IF(S238="","",IF(OR(I238=0,V238="IGEN",W238="IGEN"),0,IF(AND(K238&lt;&gt;"IGEN",L238="IGEN",U238="NEM"),0,S238)))</f>
+        <f>IF(S238="","",IF(OR(I238=0,V238="IGEN",W238="IGEN"),0,IF(AND(K238&lt;&gt;"IGEN",L238="IGEN",U238="NEM"),0,IF(AND(H238="GYES",E238&lt;1998),0,S238))))</f>
         <v/>
       </c>
       <c r="AI238" s="6">
@@ -40479,7 +40479,7 @@
         <v/>
       </c>
       <c r="AH239" s="6">
-        <f>IF(S239="","",IF(OR(I239=0,V239="IGEN",W239="IGEN"),0,IF(AND(K239&lt;&gt;"IGEN",L239="IGEN",U239="NEM"),0,S239)))</f>
+        <f>IF(S239="","",IF(OR(I239=0,V239="IGEN",W239="IGEN"),0,IF(AND(K239&lt;&gt;"IGEN",L239="IGEN",U239="NEM"),0,IF(AND(H239="GYES",E239&lt;1998),0,S239))))</f>
         <v/>
       </c>
       <c r="AI239" s="6">
@@ -40599,7 +40599,7 @@
         <v/>
       </c>
       <c r="AH240" s="6">
-        <f>IF(S240="","",IF(OR(I240=0,V240="IGEN",W240="IGEN"),0,IF(AND(K240&lt;&gt;"IGEN",L240="IGEN",U240="NEM"),0,S240)))</f>
+        <f>IF(S240="","",IF(OR(I240=0,V240="IGEN",W240="IGEN"),0,IF(AND(K240&lt;&gt;"IGEN",L240="IGEN",U240="NEM"),0,IF(AND(H240="GYES",E240&lt;1998),0,S240))))</f>
         <v/>
       </c>
       <c r="AI240" s="6">
@@ -40719,7 +40719,7 @@
         <v/>
       </c>
       <c r="AH241" s="6">
-        <f>IF(S241="","",IF(OR(I241=0,V241="IGEN",W241="IGEN"),0,IF(AND(K241&lt;&gt;"IGEN",L241="IGEN",U241="NEM"),0,S241)))</f>
+        <f>IF(S241="","",IF(OR(I241=0,V241="IGEN",W241="IGEN"),0,IF(AND(K241&lt;&gt;"IGEN",L241="IGEN",U241="NEM"),0,IF(AND(H241="GYES",E241&lt;1998),0,S241))))</f>
         <v/>
       </c>
       <c r="AI241" s="6">
@@ -40839,7 +40839,7 @@
         <v/>
       </c>
       <c r="AH242" s="6">
-        <f>IF(S242="","",IF(OR(I242=0,V242="IGEN",W242="IGEN"),0,IF(AND(K242&lt;&gt;"IGEN",L242="IGEN",U242="NEM"),0,S242)))</f>
+        <f>IF(S242="","",IF(OR(I242=0,V242="IGEN",W242="IGEN"),0,IF(AND(K242&lt;&gt;"IGEN",L242="IGEN",U242="NEM"),0,IF(AND(H242="GYES",E242&lt;1998),0,S242))))</f>
         <v/>
       </c>
       <c r="AI242" s="6">
@@ -40959,7 +40959,7 @@
         <v/>
       </c>
       <c r="AH243" s="6">
-        <f>IF(S243="","",IF(OR(I243=0,V243="IGEN",W243="IGEN"),0,IF(AND(K243&lt;&gt;"IGEN",L243="IGEN",U243="NEM"),0,S243)))</f>
+        <f>IF(S243="","",IF(OR(I243=0,V243="IGEN",W243="IGEN"),0,IF(AND(K243&lt;&gt;"IGEN",L243="IGEN",U243="NEM"),0,IF(AND(H243="GYES",E243&lt;1998),0,S243))))</f>
         <v/>
       </c>
       <c r="AI243" s="6">
@@ -41079,7 +41079,7 @@
         <v/>
       </c>
       <c r="AH244" s="6">
-        <f>IF(S244="","",IF(OR(I244=0,V244="IGEN",W244="IGEN"),0,IF(AND(K244&lt;&gt;"IGEN",L244="IGEN",U244="NEM"),0,S244)))</f>
+        <f>IF(S244="","",IF(OR(I244=0,V244="IGEN",W244="IGEN"),0,IF(AND(K244&lt;&gt;"IGEN",L244="IGEN",U244="NEM"),0,IF(AND(H244="GYES",E244&lt;1998),0,S244))))</f>
         <v/>
       </c>
       <c r="AI244" s="6">
@@ -41199,7 +41199,7 @@
         <v/>
       </c>
       <c r="AH245" s="6">
-        <f>IF(S245="","",IF(OR(I245=0,V245="IGEN",W245="IGEN"),0,IF(AND(K245&lt;&gt;"IGEN",L245="IGEN",U245="NEM"),0,S245)))</f>
+        <f>IF(S245="","",IF(OR(I245=0,V245="IGEN",W245="IGEN"),0,IF(AND(K245&lt;&gt;"IGEN",L245="IGEN",U245="NEM"),0,IF(AND(H245="GYES",E245&lt;1998),0,S245))))</f>
         <v/>
       </c>
       <c r="AI245" s="6">
@@ -41319,7 +41319,7 @@
         <v/>
       </c>
       <c r="AH246" s="6">
-        <f>IF(S246="","",IF(OR(I246=0,V246="IGEN",W246="IGEN"),0,IF(AND(K246&lt;&gt;"IGEN",L246="IGEN",U246="NEM"),0,S246)))</f>
+        <f>IF(S246="","",IF(OR(I246=0,V246="IGEN",W246="IGEN"),0,IF(AND(K246&lt;&gt;"IGEN",L246="IGEN",U246="NEM"),0,IF(AND(H246="GYES",E246&lt;1998),0,S246))))</f>
         <v/>
       </c>
       <c r="AI246" s="6">
@@ -41439,7 +41439,7 @@
         <v/>
       </c>
       <c r="AH247" s="6">
-        <f>IF(S247="","",IF(OR(I247=0,V247="IGEN",W247="IGEN"),0,IF(AND(K247&lt;&gt;"IGEN",L247="IGEN",U247="NEM"),0,S247)))</f>
+        <f>IF(S247="","",IF(OR(I247=0,V247="IGEN",W247="IGEN"),0,IF(AND(K247&lt;&gt;"IGEN",L247="IGEN",U247="NEM"),0,IF(AND(H247="GYES",E247&lt;1998),0,S247))))</f>
         <v/>
       </c>
       <c r="AI247" s="6">
@@ -41559,7 +41559,7 @@
         <v/>
       </c>
       <c r="AH248" s="6">
-        <f>IF(S248="","",IF(OR(I248=0,V248="IGEN",W248="IGEN"),0,IF(AND(K248&lt;&gt;"IGEN",L248="IGEN",U248="NEM"),0,S248)))</f>
+        <f>IF(S248="","",IF(OR(I248=0,V248="IGEN",W248="IGEN"),0,IF(AND(K248&lt;&gt;"IGEN",L248="IGEN",U248="NEM"),0,IF(AND(H248="GYES",E248&lt;1998),0,S248))))</f>
         <v/>
       </c>
       <c r="AI248" s="6">
@@ -41679,7 +41679,7 @@
         <v/>
       </c>
       <c r="AH249" s="6">
-        <f>IF(S249="","",IF(OR(I249=0,V249="IGEN",W249="IGEN"),0,IF(AND(K249&lt;&gt;"IGEN",L249="IGEN",U249="NEM"),0,S249)))</f>
+        <f>IF(S249="","",IF(OR(I249=0,V249="IGEN",W249="IGEN"),0,IF(AND(K249&lt;&gt;"IGEN",L249="IGEN",U249="NEM"),0,IF(AND(H249="GYES",E249&lt;1998),0,S249))))</f>
         <v/>
       </c>
       <c r="AI249" s="6">
@@ -41799,7 +41799,7 @@
         <v/>
       </c>
       <c r="AH250" s="6">
-        <f>IF(S250="","",IF(OR(I250=0,V250="IGEN",W250="IGEN"),0,IF(AND(K250&lt;&gt;"IGEN",L250="IGEN",U250="NEM"),0,S250)))</f>
+        <f>IF(S250="","",IF(OR(I250=0,V250="IGEN",W250="IGEN"),0,IF(AND(K250&lt;&gt;"IGEN",L250="IGEN",U250="NEM"),0,IF(AND(H250="GYES",E250&lt;1998),0,S250))))</f>
         <v/>
       </c>
       <c r="AI250" s="6">
@@ -41919,7 +41919,7 @@
         <v/>
       </c>
       <c r="AH251" s="6">
-        <f>IF(S251="","",IF(OR(I251=0,V251="IGEN",W251="IGEN"),0,IF(AND(K251&lt;&gt;"IGEN",L251="IGEN",U251="NEM"),0,S251)))</f>
+        <f>IF(S251="","",IF(OR(I251=0,V251="IGEN",W251="IGEN"),0,IF(AND(K251&lt;&gt;"IGEN",L251="IGEN",U251="NEM"),0,IF(AND(H251="GYES",E251&lt;1998),0,S251))))</f>
         <v/>
       </c>
       <c r="AI251" s="6">
@@ -42039,7 +42039,7 @@
         <v/>
       </c>
       <c r="AH252" s="6">
-        <f>IF(S252="","",IF(OR(I252=0,V252="IGEN",W252="IGEN"),0,IF(AND(K252&lt;&gt;"IGEN",L252="IGEN",U252="NEM"),0,S252)))</f>
+        <f>IF(S252="","",IF(OR(I252=0,V252="IGEN",W252="IGEN"),0,IF(AND(K252&lt;&gt;"IGEN",L252="IGEN",U252="NEM"),0,IF(AND(H252="GYES",E252&lt;1998),0,S252))))</f>
         <v/>
       </c>
       <c r="AI252" s="6">
@@ -42159,7 +42159,7 @@
         <v/>
       </c>
       <c r="AH253" s="6">
-        <f>IF(S253="","",IF(OR(I253=0,V253="IGEN",W253="IGEN"),0,IF(AND(K253&lt;&gt;"IGEN",L253="IGEN",U253="NEM"),0,S253)))</f>
+        <f>IF(S253="","",IF(OR(I253=0,V253="IGEN",W253="IGEN"),0,IF(AND(K253&lt;&gt;"IGEN",L253="IGEN",U253="NEM"),0,IF(AND(H253="GYES",E253&lt;1998),0,S253))))</f>
         <v/>
       </c>
       <c r="AI253" s="6">
@@ -42279,7 +42279,7 @@
         <v/>
       </c>
       <c r="AH254" s="6">
-        <f>IF(S254="","",IF(OR(I254=0,V254="IGEN",W254="IGEN"),0,IF(AND(K254&lt;&gt;"IGEN",L254="IGEN",U254="NEM"),0,S254)))</f>
+        <f>IF(S254="","",IF(OR(I254=0,V254="IGEN",W254="IGEN"),0,IF(AND(K254&lt;&gt;"IGEN",L254="IGEN",U254="NEM"),0,IF(AND(H254="GYES",E254&lt;1998),0,S254))))</f>
         <v/>
       </c>
       <c r="AI254" s="6">
@@ -42399,7 +42399,7 @@
         <v/>
       </c>
       <c r="AH255" s="6">
-        <f>IF(S255="","",IF(OR(I255=0,V255="IGEN",W255="IGEN"),0,IF(AND(K255&lt;&gt;"IGEN",L255="IGEN",U255="NEM"),0,S255)))</f>
+        <f>IF(S255="","",IF(OR(I255=0,V255="IGEN",W255="IGEN"),0,IF(AND(K255&lt;&gt;"IGEN",L255="IGEN",U255="NEM"),0,IF(AND(H255="GYES",E255&lt;1998),0,S255))))</f>
         <v/>
       </c>
       <c r="AI255" s="6">
@@ -42519,7 +42519,7 @@
         <v/>
       </c>
       <c r="AH256" s="6">
-        <f>IF(S256="","",IF(OR(I256=0,V256="IGEN",W256="IGEN"),0,IF(AND(K256&lt;&gt;"IGEN",L256="IGEN",U256="NEM"),0,S256)))</f>
+        <f>IF(S256="","",IF(OR(I256=0,V256="IGEN",W256="IGEN"),0,IF(AND(K256&lt;&gt;"IGEN",L256="IGEN",U256="NEM"),0,IF(AND(H256="GYES",E256&lt;1998),0,S256))))</f>
         <v/>
       </c>
       <c r="AI256" s="6">
@@ -42639,7 +42639,7 @@
         <v/>
       </c>
       <c r="AH257" s="6">
-        <f>IF(S257="","",IF(OR(I257=0,V257="IGEN",W257="IGEN"),0,IF(AND(K257&lt;&gt;"IGEN",L257="IGEN",U257="NEM"),0,S257)))</f>
+        <f>IF(S257="","",IF(OR(I257=0,V257="IGEN",W257="IGEN"),0,IF(AND(K257&lt;&gt;"IGEN",L257="IGEN",U257="NEM"),0,IF(AND(H257="GYES",E257&lt;1998),0,S257))))</f>
         <v/>
       </c>
       <c r="AI257" s="6">
@@ -42759,7 +42759,7 @@
         <v/>
       </c>
       <c r="AH258" s="6">
-        <f>IF(S258="","",IF(OR(I258=0,V258="IGEN",W258="IGEN"),0,IF(AND(K258&lt;&gt;"IGEN",L258="IGEN",U258="NEM"),0,S258)))</f>
+        <f>IF(S258="","",IF(OR(I258=0,V258="IGEN",W258="IGEN"),0,IF(AND(K258&lt;&gt;"IGEN",L258="IGEN",U258="NEM"),0,IF(AND(H258="GYES",E258&lt;1998),0,S258))))</f>
         <v/>
       </c>
       <c r="AI258" s="6">
@@ -42879,7 +42879,7 @@
         <v/>
       </c>
       <c r="AH259" s="6">
-        <f>IF(S259="","",IF(OR(I259=0,V259="IGEN",W259="IGEN"),0,IF(AND(K259&lt;&gt;"IGEN",L259="IGEN",U259="NEM"),0,S259)))</f>
+        <f>IF(S259="","",IF(OR(I259=0,V259="IGEN",W259="IGEN"),0,IF(AND(K259&lt;&gt;"IGEN",L259="IGEN",U259="NEM"),0,IF(AND(H259="GYES",E259&lt;1998),0,S259))))</f>
         <v/>
       </c>
       <c r="AI259" s="6">
@@ -42999,7 +42999,7 @@
         <v/>
       </c>
       <c r="AH260" s="6">
-        <f>IF(S260="","",IF(OR(I260=0,V260="IGEN",W260="IGEN"),0,IF(AND(K260&lt;&gt;"IGEN",L260="IGEN",U260="NEM"),0,S260)))</f>
+        <f>IF(S260="","",IF(OR(I260=0,V260="IGEN",W260="IGEN"),0,IF(AND(K260&lt;&gt;"IGEN",L260="IGEN",U260="NEM"),0,IF(AND(H260="GYES",E260&lt;1998),0,S260))))</f>
         <v/>
       </c>
       <c r="AI260" s="6">
@@ -43119,7 +43119,7 @@
         <v/>
       </c>
       <c r="AH261" s="6">
-        <f>IF(S261="","",IF(OR(I261=0,V261="IGEN",W261="IGEN"),0,IF(AND(K261&lt;&gt;"IGEN",L261="IGEN",U261="NEM"),0,S261)))</f>
+        <f>IF(S261="","",IF(OR(I261=0,V261="IGEN",W261="IGEN"),0,IF(AND(K261&lt;&gt;"IGEN",L261="IGEN",U261="NEM"),0,IF(AND(H261="GYES",E261&lt;1998),0,S261))))</f>
         <v/>
       </c>
       <c r="AI261" s="6">
@@ -43239,7 +43239,7 @@
         <v/>
       </c>
       <c r="AH262" s="6">
-        <f>IF(S262="","",IF(OR(I262=0,V262="IGEN",W262="IGEN"),0,IF(AND(K262&lt;&gt;"IGEN",L262="IGEN",U262="NEM"),0,S262)))</f>
+        <f>IF(S262="","",IF(OR(I262=0,V262="IGEN",W262="IGEN"),0,IF(AND(K262&lt;&gt;"IGEN",L262="IGEN",U262="NEM"),0,IF(AND(H262="GYES",E262&lt;1998),0,S262))))</f>
         <v/>
       </c>
       <c r="AI262" s="6">
@@ -43359,7 +43359,7 @@
         <v/>
       </c>
       <c r="AH263" s="6">
-        <f>IF(S263="","",IF(OR(I263=0,V263="IGEN",W263="IGEN"),0,IF(AND(K263&lt;&gt;"IGEN",L263="IGEN",U263="NEM"),0,S263)))</f>
+        <f>IF(S263="","",IF(OR(I263=0,V263="IGEN",W263="IGEN"),0,IF(AND(K263&lt;&gt;"IGEN",L263="IGEN",U263="NEM"),0,IF(AND(H263="GYES",E263&lt;1998),0,S263))))</f>
         <v/>
       </c>
       <c r="AI263" s="6">
@@ -43479,7 +43479,7 @@
         <v/>
       </c>
       <c r="AH264" s="6">
-        <f>IF(S264="","",IF(OR(I264=0,V264="IGEN",W264="IGEN"),0,IF(AND(K264&lt;&gt;"IGEN",L264="IGEN",U264="NEM"),0,S264)))</f>
+        <f>IF(S264="","",IF(OR(I264=0,V264="IGEN",W264="IGEN"),0,IF(AND(K264&lt;&gt;"IGEN",L264="IGEN",U264="NEM"),0,IF(AND(H264="GYES",E264&lt;1998),0,S264))))</f>
         <v/>
       </c>
       <c r="AI264" s="6">
@@ -43599,7 +43599,7 @@
         <v/>
       </c>
       <c r="AH265" s="6">
-        <f>IF(S265="","",IF(OR(I265=0,V265="IGEN",W265="IGEN"),0,IF(AND(K265&lt;&gt;"IGEN",L265="IGEN",U265="NEM"),0,S265)))</f>
+        <f>IF(S265="","",IF(OR(I265=0,V265="IGEN",W265="IGEN"),0,IF(AND(K265&lt;&gt;"IGEN",L265="IGEN",U265="NEM"),0,IF(AND(H265="GYES",E265&lt;1998),0,S265))))</f>
         <v/>
       </c>
       <c r="AI265" s="6">
@@ -43719,7 +43719,7 @@
         <v/>
       </c>
       <c r="AH266" s="6">
-        <f>IF(S266="","",IF(OR(I266=0,V266="IGEN",W266="IGEN"),0,IF(AND(K266&lt;&gt;"IGEN",L266="IGEN",U266="NEM"),0,S266)))</f>
+        <f>IF(S266="","",IF(OR(I266=0,V266="IGEN",W266="IGEN"),0,IF(AND(K266&lt;&gt;"IGEN",L266="IGEN",U266="NEM"),0,IF(AND(H266="GYES",E266&lt;1998),0,S266))))</f>
         <v/>
       </c>
       <c r="AI266" s="6">
@@ -43839,7 +43839,7 @@
         <v/>
       </c>
       <c r="AH267" s="6">
-        <f>IF(S267="","",IF(OR(I267=0,V267="IGEN",W267="IGEN"),0,IF(AND(K267&lt;&gt;"IGEN",L267="IGEN",U267="NEM"),0,S267)))</f>
+        <f>IF(S267="","",IF(OR(I267=0,V267="IGEN",W267="IGEN"),0,IF(AND(K267&lt;&gt;"IGEN",L267="IGEN",U267="NEM"),0,IF(AND(H267="GYES",E267&lt;1998),0,S267))))</f>
         <v/>
       </c>
       <c r="AI267" s="6">
@@ -43959,7 +43959,7 @@
         <v/>
       </c>
       <c r="AH268" s="6">
-        <f>IF(S268="","",IF(OR(I268=0,V268="IGEN",W268="IGEN"),0,IF(AND(K268&lt;&gt;"IGEN",L268="IGEN",U268="NEM"),0,S268)))</f>
+        <f>IF(S268="","",IF(OR(I268=0,V268="IGEN",W268="IGEN"),0,IF(AND(K268&lt;&gt;"IGEN",L268="IGEN",U268="NEM"),0,IF(AND(H268="GYES",E268&lt;1998),0,S268))))</f>
         <v/>
       </c>
       <c r="AI268" s="6">
@@ -44079,7 +44079,7 @@
         <v/>
       </c>
       <c r="AH269" s="6">
-        <f>IF(S269="","",IF(OR(I269=0,V269="IGEN",W269="IGEN"),0,IF(AND(K269&lt;&gt;"IGEN",L269="IGEN",U269="NEM"),0,S269)))</f>
+        <f>IF(S269="","",IF(OR(I269=0,V269="IGEN",W269="IGEN"),0,IF(AND(K269&lt;&gt;"IGEN",L269="IGEN",U269="NEM"),0,IF(AND(H269="GYES",E269&lt;1998),0,S269))))</f>
         <v/>
       </c>
       <c r="AI269" s="6">
@@ -44199,7 +44199,7 @@
         <v/>
       </c>
       <c r="AH270" s="6">
-        <f>IF(S270="","",IF(OR(I270=0,V270="IGEN",W270="IGEN"),0,IF(AND(K270&lt;&gt;"IGEN",L270="IGEN",U270="NEM"),0,S270)))</f>
+        <f>IF(S270="","",IF(OR(I270=0,V270="IGEN",W270="IGEN"),0,IF(AND(K270&lt;&gt;"IGEN",L270="IGEN",U270="NEM"),0,IF(AND(H270="GYES",E270&lt;1998),0,S270))))</f>
         <v/>
       </c>
       <c r="AI270" s="6">
@@ -44319,7 +44319,7 @@
         <v/>
       </c>
       <c r="AH271" s="6">
-        <f>IF(S271="","",IF(OR(I271=0,V271="IGEN",W271="IGEN"),0,IF(AND(K271&lt;&gt;"IGEN",L271="IGEN",U271="NEM"),0,S271)))</f>
+        <f>IF(S271="","",IF(OR(I271=0,V271="IGEN",W271="IGEN"),0,IF(AND(K271&lt;&gt;"IGEN",L271="IGEN",U271="NEM"),0,IF(AND(H271="GYES",E271&lt;1998),0,S271))))</f>
         <v/>
       </c>
       <c r="AI271" s="6">
@@ -44439,7 +44439,7 @@
         <v/>
       </c>
       <c r="AH272" s="6">
-        <f>IF(S272="","",IF(OR(I272=0,V272="IGEN",W272="IGEN"),0,IF(AND(K272&lt;&gt;"IGEN",L272="IGEN",U272="NEM"),0,S272)))</f>
+        <f>IF(S272="","",IF(OR(I272=0,V272="IGEN",W272="IGEN"),0,IF(AND(K272&lt;&gt;"IGEN",L272="IGEN",U272="NEM"),0,IF(AND(H272="GYES",E272&lt;1998),0,S272))))</f>
         <v/>
       </c>
       <c r="AI272" s="6">
@@ -44559,7 +44559,7 @@
         <v/>
       </c>
       <c r="AH273" s="6">
-        <f>IF(S273="","",IF(OR(I273=0,V273="IGEN",W273="IGEN"),0,IF(AND(K273&lt;&gt;"IGEN",L273="IGEN",U273="NEM"),0,S273)))</f>
+        <f>IF(S273="","",IF(OR(I273=0,V273="IGEN",W273="IGEN"),0,IF(AND(K273&lt;&gt;"IGEN",L273="IGEN",U273="NEM"),0,IF(AND(H273="GYES",E273&lt;1998),0,S273))))</f>
         <v/>
       </c>
       <c r="AI273" s="6">
@@ -44679,7 +44679,7 @@
         <v/>
       </c>
       <c r="AH274" s="6">
-        <f>IF(S274="","",IF(OR(I274=0,V274="IGEN",W274="IGEN"),0,IF(AND(K274&lt;&gt;"IGEN",L274="IGEN",U274="NEM"),0,S274)))</f>
+        <f>IF(S274="","",IF(OR(I274=0,V274="IGEN",W274="IGEN"),0,IF(AND(K274&lt;&gt;"IGEN",L274="IGEN",U274="NEM"),0,IF(AND(H274="GYES",E274&lt;1998),0,S274))))</f>
         <v/>
       </c>
       <c r="AI274" s="6">
@@ -44799,7 +44799,7 @@
         <v/>
       </c>
       <c r="AH275" s="6">
-        <f>IF(S275="","",IF(OR(I275=0,V275="IGEN",W275="IGEN"),0,IF(AND(K275&lt;&gt;"IGEN",L275="IGEN",U275="NEM"),0,S275)))</f>
+        <f>IF(S275="","",IF(OR(I275=0,V275="IGEN",W275="IGEN"),0,IF(AND(K275&lt;&gt;"IGEN",L275="IGEN",U275="NEM"),0,IF(AND(H275="GYES",E275&lt;1998),0,S275))))</f>
         <v/>
       </c>
       <c r="AI275" s="6">
@@ -44919,7 +44919,7 @@
         <v/>
       </c>
       <c r="AH276" s="6">
-        <f>IF(S276="","",IF(OR(I276=0,V276="IGEN",W276="IGEN"),0,IF(AND(K276&lt;&gt;"IGEN",L276="IGEN",U276="NEM"),0,S276)))</f>
+        <f>IF(S276="","",IF(OR(I276=0,V276="IGEN",W276="IGEN"),0,IF(AND(K276&lt;&gt;"IGEN",L276="IGEN",U276="NEM"),0,IF(AND(H276="GYES",E276&lt;1998),0,S276))))</f>
         <v/>
       </c>
       <c r="AI276" s="6">
@@ -45039,7 +45039,7 @@
         <v/>
       </c>
       <c r="AH277" s="6">
-        <f>IF(S277="","",IF(OR(I277=0,V277="IGEN",W277="IGEN"),0,IF(AND(K277&lt;&gt;"IGEN",L277="IGEN",U277="NEM"),0,S277)))</f>
+        <f>IF(S277="","",IF(OR(I277=0,V277="IGEN",W277="IGEN"),0,IF(AND(K277&lt;&gt;"IGEN",L277="IGEN",U277="NEM"),0,IF(AND(H277="GYES",E277&lt;1998),0,S277))))</f>
         <v/>
       </c>
       <c r="AI277" s="6">
@@ -45159,7 +45159,7 @@
         <v/>
       </c>
       <c r="AH278" s="6">
-        <f>IF(S278="","",IF(OR(I278=0,V278="IGEN",W278="IGEN"),0,IF(AND(K278&lt;&gt;"IGEN",L278="IGEN",U278="NEM"),0,S278)))</f>
+        <f>IF(S278="","",IF(OR(I278=0,V278="IGEN",W278="IGEN"),0,IF(AND(K278&lt;&gt;"IGEN",L278="IGEN",U278="NEM"),0,IF(AND(H278="GYES",E278&lt;1998),0,S278))))</f>
         <v/>
       </c>
       <c r="AI278" s="6">
@@ -45279,7 +45279,7 @@
         <v/>
       </c>
       <c r="AH279" s="6">
-        <f>IF(S279="","",IF(OR(I279=0,V279="IGEN",W279="IGEN"),0,IF(AND(K279&lt;&gt;"IGEN",L279="IGEN",U279="NEM"),0,S279)))</f>
+        <f>IF(S279="","",IF(OR(I279=0,V279="IGEN",W279="IGEN"),0,IF(AND(K279&lt;&gt;"IGEN",L279="IGEN",U279="NEM"),0,IF(AND(H279="GYES",E279&lt;1998),0,S279))))</f>
         <v/>
       </c>
       <c r="AI279" s="6">
@@ -45399,7 +45399,7 @@
         <v/>
       </c>
       <c r="AH280" s="6">
-        <f>IF(S280="","",IF(OR(I280=0,V280="IGEN",W280="IGEN"),0,IF(AND(K280&lt;&gt;"IGEN",L280="IGEN",U280="NEM"),0,S280)))</f>
+        <f>IF(S280="","",IF(OR(I280=0,V280="IGEN",W280="IGEN"),0,IF(AND(K280&lt;&gt;"IGEN",L280="IGEN",U280="NEM"),0,IF(AND(H280="GYES",E280&lt;1998),0,S280))))</f>
         <v/>
       </c>
       <c r="AI280" s="6">
@@ -45519,7 +45519,7 @@
         <v/>
       </c>
       <c r="AH281" s="6">
-        <f>IF(S281="","",IF(OR(I281=0,V281="IGEN",W281="IGEN"),0,IF(AND(K281&lt;&gt;"IGEN",L281="IGEN",U281="NEM"),0,S281)))</f>
+        <f>IF(S281="","",IF(OR(I281=0,V281="IGEN",W281="IGEN"),0,IF(AND(K281&lt;&gt;"IGEN",L281="IGEN",U281="NEM"),0,IF(AND(H281="GYES",E281&lt;1998),0,S281))))</f>
         <v/>
       </c>
       <c r="AI281" s="6">
@@ -45639,7 +45639,7 @@
         <v/>
       </c>
       <c r="AH282" s="6">
-        <f>IF(S282="","",IF(OR(I282=0,V282="IGEN",W282="IGEN"),0,IF(AND(K282&lt;&gt;"IGEN",L282="IGEN",U282="NEM"),0,S282)))</f>
+        <f>IF(S282="","",IF(OR(I282=0,V282="IGEN",W282="IGEN"),0,IF(AND(K282&lt;&gt;"IGEN",L282="IGEN",U282="NEM"),0,IF(AND(H282="GYES",E282&lt;1998),0,S282))))</f>
         <v/>
       </c>
       <c r="AI282" s="6">
@@ -45759,7 +45759,7 @@
         <v/>
       </c>
       <c r="AH283" s="6">
-        <f>IF(S283="","",IF(OR(I283=0,V283="IGEN",W283="IGEN"),0,IF(AND(K283&lt;&gt;"IGEN",L283="IGEN",U283="NEM"),0,S283)))</f>
+        <f>IF(S283="","",IF(OR(I283=0,V283="IGEN",W283="IGEN"),0,IF(AND(K283&lt;&gt;"IGEN",L283="IGEN",U283="NEM"),0,IF(AND(H283="GYES",E283&lt;1998),0,S283))))</f>
         <v/>
       </c>
       <c r="AI283" s="6">
@@ -45879,7 +45879,7 @@
         <v/>
       </c>
       <c r="AH284" s="6">
-        <f>IF(S284="","",IF(OR(I284=0,V284="IGEN",W284="IGEN"),0,IF(AND(K284&lt;&gt;"IGEN",L284="IGEN",U284="NEM"),0,S284)))</f>
+        <f>IF(S284="","",IF(OR(I284=0,V284="IGEN",W284="IGEN"),0,IF(AND(K284&lt;&gt;"IGEN",L284="IGEN",U284="NEM"),0,IF(AND(H284="GYES",E284&lt;1998),0,S284))))</f>
         <v/>
       </c>
       <c r="AI284" s="6">
@@ -45999,7 +45999,7 @@
         <v/>
       </c>
       <c r="AH285" s="6">
-        <f>IF(S285="","",IF(OR(I285=0,V285="IGEN",W285="IGEN"),0,IF(AND(K285&lt;&gt;"IGEN",L285="IGEN",U285="NEM"),0,S285)))</f>
+        <f>IF(S285="","",IF(OR(I285=0,V285="IGEN",W285="IGEN"),0,IF(AND(K285&lt;&gt;"IGEN",L285="IGEN",U285="NEM"),0,IF(AND(H285="GYES",E285&lt;1998),0,S285))))</f>
         <v/>
       </c>
       <c r="AI285" s="6">
@@ -46119,7 +46119,7 @@
         <v/>
       </c>
       <c r="AH286" s="6">
-        <f>IF(S286="","",IF(OR(I286=0,V286="IGEN",W286="IGEN"),0,IF(AND(K286&lt;&gt;"IGEN",L286="IGEN",U286="NEM"),0,S286)))</f>
+        <f>IF(S286="","",IF(OR(I286=0,V286="IGEN",W286="IGEN"),0,IF(AND(K286&lt;&gt;"IGEN",L286="IGEN",U286="NEM"),0,IF(AND(H286="GYES",E286&lt;1998),0,S286))))</f>
         <v/>
       </c>
       <c r="AI286" s="6">
@@ -46239,7 +46239,7 @@
         <v/>
       </c>
       <c r="AH287" s="6">
-        <f>IF(S287="","",IF(OR(I287=0,V287="IGEN",W287="IGEN"),0,IF(AND(K287&lt;&gt;"IGEN",L287="IGEN",U287="NEM"),0,S287)))</f>
+        <f>IF(S287="","",IF(OR(I287=0,V287="IGEN",W287="IGEN"),0,IF(AND(K287&lt;&gt;"IGEN",L287="IGEN",U287="NEM"),0,IF(AND(H287="GYES",E287&lt;1998),0,S287))))</f>
         <v/>
       </c>
       <c r="AI287" s="6">
@@ -46359,7 +46359,7 @@
         <v/>
       </c>
       <c r="AH288" s="6">
-        <f>IF(S288="","",IF(OR(I288=0,V288="IGEN",W288="IGEN"),0,IF(AND(K288&lt;&gt;"IGEN",L288="IGEN",U288="NEM"),0,S288)))</f>
+        <f>IF(S288="","",IF(OR(I288=0,V288="IGEN",W288="IGEN"),0,IF(AND(K288&lt;&gt;"IGEN",L288="IGEN",U288="NEM"),0,IF(AND(H288="GYES",E288&lt;1998),0,S288))))</f>
         <v/>
       </c>
       <c r="AI288" s="6">
@@ -46479,7 +46479,7 @@
         <v/>
       </c>
       <c r="AH289" s="6">
-        <f>IF(S289="","",IF(OR(I289=0,V289="IGEN",W289="IGEN"),0,IF(AND(K289&lt;&gt;"IGEN",L289="IGEN",U289="NEM"),0,S289)))</f>
+        <f>IF(S289="","",IF(OR(I289=0,V289="IGEN",W289="IGEN"),0,IF(AND(K289&lt;&gt;"IGEN",L289="IGEN",U289="NEM"),0,IF(AND(H289="GYES",E289&lt;1998),0,S289))))</f>
         <v/>
       </c>
       <c r="AI289" s="6">
@@ -46599,7 +46599,7 @@
         <v/>
       </c>
       <c r="AH290" s="6">
-        <f>IF(S290="","",IF(OR(I290=0,V290="IGEN",W290="IGEN"),0,IF(AND(K290&lt;&gt;"IGEN",L290="IGEN",U290="NEM"),0,S290)))</f>
+        <f>IF(S290="","",IF(OR(I290=0,V290="IGEN",W290="IGEN"),0,IF(AND(K290&lt;&gt;"IGEN",L290="IGEN",U290="NEM"),0,IF(AND(H290="GYES",E290&lt;1998),0,S290))))</f>
         <v/>
       </c>
       <c r="AI290" s="6">
@@ -46719,7 +46719,7 @@
         <v/>
       </c>
       <c r="AH291" s="6">
-        <f>IF(S291="","",IF(OR(I291=0,V291="IGEN",W291="IGEN"),0,IF(AND(K291&lt;&gt;"IGEN",L291="IGEN",U291="NEM"),0,S291)))</f>
+        <f>IF(S291="","",IF(OR(I291=0,V291="IGEN",W291="IGEN"),0,IF(AND(K291&lt;&gt;"IGEN",L291="IGEN",U291="NEM"),0,IF(AND(H291="GYES",E291&lt;1998),0,S291))))</f>
         <v/>
       </c>
       <c r="AI291" s="6">
@@ -46839,7 +46839,7 @@
         <v/>
       </c>
       <c r="AH292" s="6">
-        <f>IF(S292="","",IF(OR(I292=0,V292="IGEN",W292="IGEN"),0,IF(AND(K292&lt;&gt;"IGEN",L292="IGEN",U292="NEM"),0,S292)))</f>
+        <f>IF(S292="","",IF(OR(I292=0,V292="IGEN",W292="IGEN"),0,IF(AND(K292&lt;&gt;"IGEN",L292="IGEN",U292="NEM"),0,IF(AND(H292="GYES",E292&lt;1998),0,S292))))</f>
         <v/>
       </c>
       <c r="AI292" s="6">
@@ -46959,7 +46959,7 @@
         <v/>
       </c>
       <c r="AH293" s="6">
-        <f>IF(S293="","",IF(OR(I293=0,V293="IGEN",W293="IGEN"),0,IF(AND(K293&lt;&gt;"IGEN",L293="IGEN",U293="NEM"),0,S293)))</f>
+        <f>IF(S293="","",IF(OR(I293=0,V293="IGEN",W293="IGEN"),0,IF(AND(K293&lt;&gt;"IGEN",L293="IGEN",U293="NEM"),0,IF(AND(H293="GYES",E293&lt;1998),0,S293))))</f>
         <v/>
       </c>
       <c r="AI293" s="6">
@@ -47079,7 +47079,7 @@
         <v/>
       </c>
       <c r="AH294" s="6">
-        <f>IF(S294="","",IF(OR(I294=0,V294="IGEN",W294="IGEN"),0,IF(AND(K294&lt;&gt;"IGEN",L294="IGEN",U294="NEM"),0,S294)))</f>
+        <f>IF(S294="","",IF(OR(I294=0,V294="IGEN",W294="IGEN"),0,IF(AND(K294&lt;&gt;"IGEN",L294="IGEN",U294="NEM"),0,IF(AND(H294="GYES",E294&lt;1998),0,S294))))</f>
         <v/>
       </c>
       <c r="AI294" s="6">
@@ -47199,7 +47199,7 @@
         <v/>
       </c>
       <c r="AH295" s="6">
-        <f>IF(S295="","",IF(OR(I295=0,V295="IGEN",W295="IGEN"),0,IF(AND(K295&lt;&gt;"IGEN",L295="IGEN",U295="NEM"),0,S295)))</f>
+        <f>IF(S295="","",IF(OR(I295=0,V295="IGEN",W295="IGEN"),0,IF(AND(K295&lt;&gt;"IGEN",L295="IGEN",U295="NEM"),0,IF(AND(H295="GYES",E295&lt;1998),0,S295))))</f>
         <v/>
       </c>
       <c r="AI295" s="6">
@@ -47319,7 +47319,7 @@
         <v/>
       </c>
       <c r="AH296" s="6">
-        <f>IF(S296="","",IF(OR(I296=0,V296="IGEN",W296="IGEN"),0,IF(AND(K296&lt;&gt;"IGEN",L296="IGEN",U296="NEM"),0,S296)))</f>
+        <f>IF(S296="","",IF(OR(I296=0,V296="IGEN",W296="IGEN"),0,IF(AND(K296&lt;&gt;"IGEN",L296="IGEN",U296="NEM"),0,IF(AND(H296="GYES",E296&lt;1998),0,S296))))</f>
         <v/>
       </c>
       <c r="AI296" s="6">
@@ -47439,7 +47439,7 @@
         <v/>
       </c>
       <c r="AH297" s="6">
-        <f>IF(S297="","",IF(OR(I297=0,V297="IGEN",W297="IGEN"),0,IF(AND(K297&lt;&gt;"IGEN",L297="IGEN",U297="NEM"),0,S297)))</f>
+        <f>IF(S297="","",IF(OR(I297=0,V297="IGEN",W297="IGEN"),0,IF(AND(K297&lt;&gt;"IGEN",L297="IGEN",U297="NEM"),0,IF(AND(H297="GYES",E297&lt;1998),0,S297))))</f>
         <v/>
       </c>
       <c r="AI297" s="6">
@@ -47559,7 +47559,7 @@
         <v/>
       </c>
       <c r="AH298" s="6">
-        <f>IF(S298="","",IF(OR(I298=0,V298="IGEN",W298="IGEN"),0,IF(AND(K298&lt;&gt;"IGEN",L298="IGEN",U298="NEM"),0,S298)))</f>
+        <f>IF(S298="","",IF(OR(I298=0,V298="IGEN",W298="IGEN"),0,IF(AND(K298&lt;&gt;"IGEN",L298="IGEN",U298="NEM"),0,IF(AND(H298="GYES",E298&lt;1998),0,S298))))</f>
         <v/>
       </c>
       <c r="AI298" s="6">
@@ -47679,7 +47679,7 @@
         <v/>
       </c>
       <c r="AH299" s="6">
-        <f>IF(S299="","",IF(OR(I299=0,V299="IGEN",W299="IGEN"),0,IF(AND(K299&lt;&gt;"IGEN",L299="IGEN",U299="NEM"),0,S299)))</f>
+        <f>IF(S299="","",IF(OR(I299=0,V299="IGEN",W299="IGEN"),0,IF(AND(K299&lt;&gt;"IGEN",L299="IGEN",U299="NEM"),0,IF(AND(H299="GYES",E299&lt;1998),0,S299))))</f>
         <v/>
       </c>
       <c r="AI299" s="6">
@@ -47799,7 +47799,7 @@
         <v/>
       </c>
       <c r="AH300" s="6">
-        <f>IF(S300="","",IF(OR(I300=0,V300="IGEN",W300="IGEN"),0,IF(AND(K300&lt;&gt;"IGEN",L300="IGEN",U300="NEM"),0,S300)))</f>
+        <f>IF(S300="","",IF(OR(I300=0,V300="IGEN",W300="IGEN"),0,IF(AND(K300&lt;&gt;"IGEN",L300="IGEN",U300="NEM"),0,IF(AND(H300="GYES",E300&lt;1998),0,S300))))</f>
         <v/>
       </c>
       <c r="AI300" s="6">
@@ -47919,7 +47919,7 @@
         <v/>
       </c>
       <c r="AH301" s="6">
-        <f>IF(S301="","",IF(OR(I301=0,V301="IGEN",W301="IGEN"),0,IF(AND(K301&lt;&gt;"IGEN",L301="IGEN",U301="NEM"),0,S301)))</f>
+        <f>IF(S301="","",IF(OR(I301=0,V301="IGEN",W301="IGEN"),0,IF(AND(K301&lt;&gt;"IGEN",L301="IGEN",U301="NEM"),0,IF(AND(H301="GYES",E301&lt;1998),0,S301))))</f>
         <v/>
       </c>
       <c r="AI301" s="6">
@@ -48039,7 +48039,7 @@
         <v/>
       </c>
       <c r="AH302" s="6">
-        <f>IF(S302="","",IF(OR(I302=0,V302="IGEN",W302="IGEN"),0,IF(AND(K302&lt;&gt;"IGEN",L302="IGEN",U302="NEM"),0,S302)))</f>
+        <f>IF(S302="","",IF(OR(I302=0,V302="IGEN",W302="IGEN"),0,IF(AND(K302&lt;&gt;"IGEN",L302="IGEN",U302="NEM"),0,IF(AND(H302="GYES",E302&lt;1998),0,S302))))</f>
         <v/>
       </c>
       <c r="AI302" s="6">
@@ -48159,7 +48159,7 @@
         <v/>
       </c>
       <c r="AH303" s="6">
-        <f>IF(S303="","",IF(OR(I303=0,V303="IGEN",W303="IGEN"),0,IF(AND(K303&lt;&gt;"IGEN",L303="IGEN",U303="NEM"),0,S303)))</f>
+        <f>IF(S303="","",IF(OR(I303=0,V303="IGEN",W303="IGEN"),0,IF(AND(K303&lt;&gt;"IGEN",L303="IGEN",U303="NEM"),0,IF(AND(H303="GYES",E303&lt;1998),0,S303))))</f>
         <v/>
       </c>
       <c r="AI303" s="6">
@@ -48279,7 +48279,7 @@
         <v/>
       </c>
       <c r="AH304" s="6">
-        <f>IF(S304="","",IF(OR(I304=0,V304="IGEN",W304="IGEN"),0,IF(AND(K304&lt;&gt;"IGEN",L304="IGEN",U304="NEM"),0,S304)))</f>
+        <f>IF(S304="","",IF(OR(I304=0,V304="IGEN",W304="IGEN"),0,IF(AND(K304&lt;&gt;"IGEN",L304="IGEN",U304="NEM"),0,IF(AND(H304="GYES",E304&lt;1998),0,S304))))</f>
         <v/>
       </c>
       <c r="AI304" s="6">

</xml_diff>